<commit_message>
docs(qa): add checklist rows for the UX polish pass
Fifteen rows in a new 2.10 section on the QA sheet, styled from the 2.9
rows so the counters and conditional formatting keep working.

They are the cases a person has to check because nothing automated can:
the focus actually moving, the ring actually painting, reduced motion
actually being honoured, and a mission with no notes rendering without a
heading over blank space on all three surfaces.

Also two lines of copy that still promised a brief the product no longer
requires — the guidelines said to follow the builder instructions, and
the landing page said every mission ships with a brief from the builder.
Both now name the test case, which is the thing that is actually always
there.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rodskbpmg84yDZUZtkK4RN
</commit_message>
<xml_diff>
--- a/TownHall_Checklist (1).xlsx
+++ b/TownHall_Checklist (1).xlsx
@@ -2683,7 +2683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:E93"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4167,6 +4167,298 @@
         </is>
       </c>
       <c r="E76" s="7" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2.10 UX polish — error focus, focus rings, optional notes, audit fields</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="n"/>
+      <c r="B79" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.10-1</t>
+        </is>
+      </c>
+      <c r="C79" s="9" t="inlineStr">
+        <is>
+          <t>Submitting any form with a required field empty scrolls that field into view and focuses it — try /dashboard/new empty, and the mission form with a blank test step.</t>
+        </is>
+      </c>
+      <c r="D79" s="23" t="inlineStr">
+        <is>
+          <t>New in the UX polish pass</t>
+        </is>
+      </c>
+      <c r="E79" s="7" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="n"/>
+      <c r="B80" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.10-2</t>
+        </is>
+      </c>
+      <c r="C80" s="9" t="inlineStr">
+        <is>
+          <t>The mission form sends you to the FIRST error on the page, not the first one the schema found — a blank step beats the notes below it.</t>
+        </is>
+      </c>
+      <c r="D80" s="23" t="inlineStr">
+        <is>
+          <t>New in the UX polish pass</t>
+        </is>
+      </c>
+      <c r="E80" s="7" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="n"/>
+      <c r="B81" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.10-3</t>
+        </is>
+      </c>
+      <c r="C81" s="9" t="inlineStr">
+        <is>
+          <t>Submitting twice without fixing anything moves you both times.</t>
+        </is>
+      </c>
+      <c r="D81" s="23" t="inlineStr">
+        <is>
+          <t>New in the UX polish pass</t>
+        </is>
+      </c>
+      <c r="E81" s="7" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="n"/>
+      <c r="B82" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.10-4</t>
+        </is>
+      </c>
+      <c r="C82" s="9" t="inlineStr">
+        <is>
+          <t>Tab through the sidebar with the keyboard: the builder/tester switch and every nav item show a voltage focus ring, against both dark surfaces.</t>
+        </is>
+      </c>
+      <c r="D82" s="23" t="inlineStr">
+        <is>
+          <t>New in the UX polish pass</t>
+        </is>
+      </c>
+      <c r="E82" s="7" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="n"/>
+      <c r="B83" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.10-5</t>
+        </is>
+      </c>
+      <c r="C83" s="9" t="inlineStr">
+        <is>
+          <t>With OS 'reduce motion' on, the jump to an errored field is instant rather than smooth.</t>
+        </is>
+      </c>
+      <c r="D83" s="23" t="inlineStr">
+        <is>
+          <t>New in the UX polish pass</t>
+        </is>
+      </c>
+      <c r="E83" s="7" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="n"/>
+      <c r="B84" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.10-6</t>
+        </is>
+      </c>
+      <c r="C84" s="9" t="inlineStr">
+        <is>
+          <t>An incomplete audit log names the step: 'Step 4 needs an answer.', scrolls to that card, focuses its first empty field, and outlines it.</t>
+        </is>
+      </c>
+      <c r="D84" s="23" t="inlineStr">
+        <is>
+          <t>New in the UX polish pass</t>
+        </is>
+      </c>
+      <c r="E84" s="7" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="n"/>
+      <c r="B85" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.10-7</t>
+        </is>
+      </c>
+      <c r="C85" s="9" t="inlineStr">
+        <is>
+          <t>Create a mission with 'Add notes for testers' unchecked — it saves, and the mission renders with no empty heading on the tester page, the builder page and /admin.</t>
+        </is>
+      </c>
+      <c r="D85" s="23" t="inlineStr">
+        <is>
+          <t>New in the UX polish pass</t>
+        </is>
+      </c>
+      <c r="E85" s="7" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="n"/>
+      <c r="B86" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.10-8</t>
+        </is>
+      </c>
+      <c r="C86" s="9" t="inlineStr">
+        <is>
+          <t>Editing a mission that already has notes opens with the box checked and the text intact.</t>
+        </is>
+      </c>
+      <c r="D86" s="23" t="inlineStr">
+        <is>
+          <t>New in the UX polish pass</t>
+        </is>
+      </c>
+      <c r="E86" s="7" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="n"/>
+      <c r="B87" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.10-9</t>
+        </is>
+      </c>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>Notes with 5 characters are refused, with a message offering both ways out.</t>
+        </is>
+      </c>
+      <c r="D87" s="23" t="inlineStr">
+        <is>
+          <t>New in the UX polish pass</t>
+        </is>
+      </c>
+      <c r="E87" s="7" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="3" t="n"/>
+      <c r="B88" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.10-10</t>
+        </is>
+      </c>
+      <c r="C88" s="9" t="inlineStr">
+        <is>
+          <t>A step marked Pass is not asked what actually happened — only what you expected.</t>
+        </is>
+      </c>
+      <c r="D88" s="23" t="inlineStr">
+        <is>
+          <t>New in the UX polish pass</t>
+        </is>
+      </c>
+      <c r="E88" s="7" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="n"/>
+      <c r="B89" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.10-11</t>
+        </is>
+      </c>
+      <c r="C89" s="9" t="inlineStr">
+        <is>
+          <t>A step marked Blocked IS asked what happened, for a summary and for steps to reproduce, and all three are required to submit.</t>
+        </is>
+      </c>
+      <c r="D89" s="23" t="inlineStr">
+        <is>
+          <t>New in the UX polish pass</t>
+        </is>
+      </c>
+      <c r="E89" s="7" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="n"/>
+      <c r="B90" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.10-12</t>
+        </is>
+      </c>
+      <c r="C90" s="9" t="inlineStr">
+        <is>
+          <t>A submission containing a passing step renders on the builder side with no bare 'Actual:' label.</t>
+        </is>
+      </c>
+      <c r="D90" s="23" t="inlineStr">
+        <is>
+          <t>New in the UX polish pass</t>
+        </is>
+      </c>
+      <c r="E90" s="7" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="3" t="n"/>
+      <c r="B91" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.10-13</t>
+        </is>
+      </c>
+      <c r="C91" s="9" t="inlineStr">
+        <is>
+          <t>The tester tour's first step points at the test case and reads correctly on a mission with no notes.</t>
+        </is>
+      </c>
+      <c r="D91" s="23" t="inlineStr">
+        <is>
+          <t>New in the UX polish pass</t>
+        </is>
+      </c>
+      <c r="E91" s="7" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="3" t="n"/>
+      <c r="B92" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.10-14</t>
+        </is>
+      </c>
+      <c r="C92" s="9" t="inlineStr">
+        <is>
+          <t>The screenshot section reads 'Screenshots of Your Test'; the builder side reads 'TEST SCREENSHOTS'; no 'Proof of Visit' anywhere.</t>
+        </is>
+      </c>
+      <c r="D92" s="23" t="inlineStr">
+        <is>
+          <t>New in the UX polish pass</t>
+        </is>
+      </c>
+      <c r="E92" s="7" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="n"/>
+      <c r="B93" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.10-15</t>
+        </is>
+      </c>
+      <c r="C93" s="9" t="inlineStr">
+        <is>
+          <t>There is one button in the tester's CTA row, and a line under it saying answers save on this device. Reload mid-log — answers restored.</t>
+        </is>
+      </c>
+      <c r="D93" s="23" t="inlineStr">
+        <is>
+          <t>New in the UX polish pass</t>
+        </is>
+      </c>
+      <c r="E93" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>

<commit_message>
docs: record active-role input and phone/country rule
CLAUDE.md now says Settings components require the active account type,
that role redirects go through landingFor(), and how the phone/country
check works and where its traps are. The QA checklist gains section
2.11 for the three fixes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TownHall_Checklist (1).xlsx
+++ b/TownHall_Checklist (1).xlsx
@@ -2683,7 +2683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E93"/>
+  <dimension ref="A1:E103"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2875,6 +2875,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="19.5" customHeight="1">
       <c r="A11" s="39" t="inlineStr">
         <is>
@@ -3013,6 +3014,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="19.5" customHeight="1">
       <c r="A18" s="39" t="inlineStr">
         <is>
@@ -3182,6 +3184,7 @@
         </is>
       </c>
     </row>
+    <row r="25"/>
     <row r="26" ht="19.5" customHeight="1">
       <c r="A26" s="39" t="inlineStr">
         <is>
@@ -3343,6 +3346,7 @@
         </is>
       </c>
     </row>
+    <row r="33"/>
     <row r="34" ht="19.5" customHeight="1">
       <c r="A34" s="39" t="inlineStr">
         <is>
@@ -3431,6 +3435,7 @@
         </is>
       </c>
     </row>
+    <row r="38"/>
     <row r="39" ht="19.5" customHeight="1">
       <c r="A39" s="39" t="inlineStr">
         <is>
@@ -3515,6 +3520,7 @@
         </is>
       </c>
     </row>
+    <row r="43"/>
     <row r="44" ht="19.5" customHeight="1">
       <c r="A44" s="39" t="inlineStr">
         <is>
@@ -3761,6 +3767,7 @@
         </is>
       </c>
     </row>
+    <row r="54"/>
     <row r="55" ht="19.5" customHeight="1">
       <c r="A55" s="39" t="inlineStr">
         <is>
@@ -3876,6 +3883,7 @@
         </is>
       </c>
     </row>
+    <row r="60"/>
     <row r="61">
       <c r="A61" s="39" t="inlineStr">
         <is>
@@ -4168,6 +4176,7 @@
       </c>
       <c r="E76" s="7" t="n"/>
     </row>
+    <row r="77"/>
     <row r="78">
       <c r="A78" s="39" t="inlineStr">
         <is>
@@ -4459,6 +4468,166 @@
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr"/>
+    </row>
+    <row r="94"/>
+    <row r="95">
+      <c r="A95" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2.11 Bug fix round 1 — found on an Android phone</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="n"/>
+      <c r="B96" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.11-1</t>
+        </is>
+      </c>
+      <c r="C96" s="9" t="inlineStr">
+        <is>
+          <t>On a tester account, Settings → Account reads "Builder account" and the button says "Add builder account" (or "Switch to builder account" if you hold both) — never "tester". Tapping Switch lands on the dashboard.</t>
+        </is>
+      </c>
+      <c r="D96" s="23" t="inlineStr">
+        <is>
+          <t>New in bug fix round 1</t>
+        </is>
+      </c>
+      <c r="E96" s="7" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="n"/>
+      <c r="B97" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.11-2</t>
+        </is>
+      </c>
+      <c r="C97" s="9" t="inlineStr">
+        <is>
+          <t>On a builder account, the same section still reads "Tester account" with the original copy about earning reports.</t>
+        </is>
+      </c>
+      <c r="D97" s="23" t="inlineStr">
+        <is>
+          <t>New in bug fix round 1</t>
+        </is>
+      </c>
+      <c r="E97" s="7" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="3" t="n"/>
+      <c r="B98" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.11-3</t>
+        </is>
+      </c>
+      <c r="C98" s="9" t="inlineStr">
+        <is>
+          <t>On a tester account, Settings has no Plan tab, and /settings?tab=plan opens Profile.</t>
+        </is>
+      </c>
+      <c r="D98" s="23" t="inlineStr">
+        <is>
+          <t>New in bug fix round 1</t>
+        </is>
+      </c>
+      <c r="E98" s="7" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="3" t="n"/>
+      <c r="B99" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.11-4</t>
+        </is>
+      </c>
+      <c r="C99" s="9" t="inlineStr">
+        <is>
+          <t>As a new user on /choose-account at 360px, tapping a card changes its label to "Creating…" at once and BOTH cards lock; tapping the other card does nothing.</t>
+        </is>
+      </c>
+      <c r="D99" s="23" t="inlineStr">
+        <is>
+          <t>New in bug fix round 1</t>
+        </is>
+      </c>
+      <c r="E99" s="7" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="3" t="n"/>
+      <c r="B100" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.11-5</t>
+        </is>
+      </c>
+      <c r="C100" s="9" t="inlineStr">
+        <is>
+          <t>After creating an account you land straight on the profile form (/verify/[role]) — a loading skeleton shows while it opens, and the dashboard never flashes first.</t>
+        </is>
+      </c>
+      <c r="D100" s="23" t="inlineStr">
+        <is>
+          <t>New in bug fix round 1</t>
+        </is>
+      </c>
+      <c r="E100" s="7" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="3" t="n"/>
+      <c r="B101" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.11-6</t>
+        </is>
+      </c>
+      <c r="C101" s="9" t="inlineStr">
+        <is>
+          <t>On the verification form, selecting Botswana shows a +267 example under Phone; changing the country updates it.</t>
+        </is>
+      </c>
+      <c r="D101" s="23" t="inlineStr">
+        <is>
+          <t>New in bug fix round 1</t>
+        </is>
+      </c>
+      <c r="E101" s="7" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="n"/>
+      <c r="B102" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.11-7</t>
+        </is>
+      </c>
+      <c r="C102" s="9" t="inlineStr">
+        <is>
+          <t>With Botswana selected, a Nigerian number (+234 801 234 5678) is rejected on the Phone field with a message naming Botswana.</t>
+        </is>
+      </c>
+      <c r="D102" s="23" t="inlineStr">
+        <is>
+          <t>New in bug fix round 1</t>
+        </is>
+      </c>
+      <c r="E102" s="7" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="3" t="n"/>
+      <c r="B103" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.11-8</t>
+        </is>
+      </c>
+      <c r="C103" s="9" t="inlineStr">
+        <is>
+          <t>A +1 number is accepted with United States selected and with Canada selected.</t>
+        </is>
+      </c>
+      <c r="D103" s="23" t="inlineStr">
+        <is>
+          <t>New in bug fix round 1</t>
+        </is>
+      </c>
+      <c r="E103" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>

<commit_message>
docs: record the ui_design rule and the round-1 additions
The spec gains sections 4 and 5, including why ui_design inverts
20260907_01 and where the design labels do and do not follow. CLAUDE.md
records the ui_design exception to the audit-log pass rule and that
role-awareness applies inside the Settings tabs too. The QA checklist
gains rows for both.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TownHall_Checklist (1).xlsx
+++ b/TownHall_Checklist (1).xlsx
@@ -2683,7 +2683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E103"/>
+  <dimension ref="A1:E108"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2875,7 +2875,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="19.5" customHeight="1">
       <c r="A11" s="39" t="inlineStr">
         <is>
@@ -3014,7 +3013,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="19.5" customHeight="1">
       <c r="A18" s="39" t="inlineStr">
         <is>
@@ -3184,7 +3182,6 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
     <row r="26" ht="19.5" customHeight="1">
       <c r="A26" s="39" t="inlineStr">
         <is>
@@ -3346,7 +3343,6 @@
         </is>
       </c>
     </row>
-    <row r="33"/>
     <row r="34" ht="19.5" customHeight="1">
       <c r="A34" s="39" t="inlineStr">
         <is>
@@ -3435,7 +3431,6 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
     <row r="39" ht="19.5" customHeight="1">
       <c r="A39" s="39" t="inlineStr">
         <is>
@@ -3520,7 +3515,6 @@
         </is>
       </c>
     </row>
-    <row r="43"/>
     <row r="44" ht="19.5" customHeight="1">
       <c r="A44" s="39" t="inlineStr">
         <is>
@@ -3767,7 +3761,6 @@
         </is>
       </c>
     </row>
-    <row r="54"/>
     <row r="55" ht="19.5" customHeight="1">
       <c r="A55" s="39" t="inlineStr">
         <is>
@@ -3883,7 +3876,6 @@
         </is>
       </c>
     </row>
-    <row r="60"/>
     <row r="61">
       <c r="A61" s="39" t="inlineStr">
         <is>
@@ -4176,7 +4168,6 @@
       </c>
       <c r="E76" s="7" t="n"/>
     </row>
-    <row r="77"/>
     <row r="78">
       <c r="A78" s="39" t="inlineStr">
         <is>
@@ -4469,7 +4460,6 @@
       </c>
       <c r="E93" s="7" t="inlineStr"/>
     </row>
-    <row r="94"/>
     <row r="95">
       <c r="A95" s="39" t="inlineStr">
         <is>
@@ -4628,6 +4618,101 @@
         </is>
       </c>
       <c r="E103" s="7" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="3" t="n"/>
+      <c r="B104" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.11-9</t>
+        </is>
+      </c>
+      <c r="C104" s="9" t="inlineStr">
+        <is>
+          <t>On a tester account, Settings → Account has no "Export your data" section; on a builder with no feedback it is still there with "Nothing to export yet".</t>
+        </is>
+      </c>
+      <c r="D104" s="23" t="inlineStr">
+        <is>
+          <t>New in bug fix round 1</t>
+        </is>
+      </c>
+      <c r="E104" s="7" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="3" t="n"/>
+      <c r="B105" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.11-10</t>
+        </is>
+      </c>
+      <c r="C105" s="9" t="inlineStr">
+        <is>
+          <t>On a tester account, Settings → Activity reads "Your testing" with Reports written, Approved and Average rating — no Reports received, no Give / take, nothing about pay. An unrated tester sees "—".</t>
+        </is>
+      </c>
+      <c r="D105" s="23" t="inlineStr">
+        <is>
+          <t>New in bug fix round 1</t>
+        </is>
+      </c>
+      <c r="E105" s="7" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="3" t="n"/>
+      <c r="B106" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.11-11</t>
+        </is>
+      </c>
+      <c r="C106" s="9" t="inlineStr">
+        <is>
+          <t>On a UI Design mission, each step asks "What you saw" first, and the choices read Clear / Unclear / Couldn't tell under "Did the builder's expectation hold?".</t>
+        </is>
+      </c>
+      <c r="D106" s="23" t="inlineStr">
+        <is>
+          <t>New in bug fix round 1</t>
+        </is>
+      </c>
+      <c r="E106" s="7" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="n"/>
+      <c r="B107" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.11-12</t>
+        </is>
+      </c>
+      <c r="C107" s="9" t="inlineStr">
+        <is>
+          <t>On a UI Design mission, marking Clear with an empty or very short description cannot be submitted — the form names the step and focuses "What you saw".</t>
+        </is>
+      </c>
+      <c r="D107" s="23" t="inlineStr">
+        <is>
+          <t>New in bug fix round 1</t>
+        </is>
+      </c>
+      <c r="E107" s="7" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="n"/>
+      <c r="B108" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.11-13</t>
+        </is>
+      </c>
+      <c r="C108" s="9" t="inlineStr">
+        <is>
+          <t>On a Process Flow or Component mission, the choices still read Pass / Fail / Blocked and a Pass with nothing written still submits.</t>
+        </is>
+      </c>
+      <c r="D108" s="23" t="inlineStr">
+        <is>
+          <t>New in bug fix round 1</t>
+        </is>
+      </c>
+      <c r="E108" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>

<commit_message>
docs: record ai_usage_events and the metering QA row
CLAUDE.md gains the table, marked service-role only and a cost record
rather than a quota ledger. The QA checklist gains section 2.12: a
submission still succeeds when the metering insert fails.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TownHall_Checklist (1).xlsx
+++ b/TownHall_Checklist (1).xlsx
@@ -2683,7 +2683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E108"/>
+  <dimension ref="A1:E112"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4713,6 +4713,51 @@
         </is>
       </c>
       <c r="E108" s="7" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2.12 AI shadow metering — ai_usage_events</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="n"/>
+      <c r="B111" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.12-1</t>
+        </is>
+      </c>
+      <c r="C111" s="9" t="inlineStr">
+        <is>
+          <t>With the ai_usage_events insert failing (table renamed or revoked on staging), submit a test: the submission saves, the builder sees it, and the AI summary still populates. One "[recordAiUsage]" line in the server log.</t>
+        </is>
+      </c>
+      <c r="D111" s="23" t="inlineStr">
+        <is>
+          <t>New in AI shadow metering</t>
+        </is>
+      </c>
+      <c r="E111" s="7" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="3" t="n"/>
+      <c r="B112" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.12-2</t>
+        </is>
+      </c>
+      <c r="C112" s="9" t="inlineStr">
+        <is>
+          <t>Submit a test normally: exactly one ai_usage_events row, status succeeded, with token counts and a cost; /admin/ai-reports shows it in this month's spend. With Gemini unavailable, the row is status failed with the error.</t>
+        </is>
+      </c>
+      <c r="D112" s="23" t="inlineStr">
+        <is>
+          <t>New in AI shadow metering</t>
+        </is>
+      </c>
+      <c r="E112" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>

<commit_message>
docs: record the ledger and publish-time enforcement
The not-enforced warnings in lib/plans.ts and /pricing come down.
QA rows for publish, cap, release, grant and the admin tile.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TownHall_Checklist (1).xlsx
+++ b/TownHall_Checklist (1).xlsx
@@ -2683,7 +2683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E108"/>
+  <dimension ref="A1:E118"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4713,6 +4713,184 @@
         </is>
       </c>
       <c r="E108" s="7" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2.12 Report allowance — publish, cap, release</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="3" t="n"/>
+      <c r="B110" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.12-1</t>
+        </is>
+      </c>
+      <c r="C110" s="9" t="inlineStr">
+        <is>
+          <t>A brand-new Community builder publishes a mission → it goes live open to 3 testers, and the mission page says it is open to 3 testers with a "Write a report for someone else" link.</t>
+        </is>
+      </c>
+      <c r="D110" s="23" t="inlineStr">
+        <is>
+          <t>New in report allowance</t>
+        </is>
+      </c>
+      <c r="E110" s="7" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="n"/>
+      <c r="B111" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.12-2</t>
+        </is>
+      </c>
+      <c r="C111" s="9" t="inlineStr">
+        <is>
+          <t>The same builder publishes a second mission → it stays a draft, and the mission page says there are no reports available, with links to write a report and to get in touch about Pro.</t>
+        </is>
+      </c>
+      <c r="D111" s="23" t="inlineStr">
+        <is>
+          <t>New in report allowance</t>
+        </is>
+      </c>
+      <c r="E111" s="7" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="3" t="n"/>
+      <c r="B112" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.12-3</t>
+        </is>
+      </c>
+      <c r="C112" s="9" t="inlineStr">
+        <is>
+          <t>The builder switches to tester, submits a report on someone else's mission, switches back → the new-mission form now says "You have 1 report available".</t>
+        </is>
+      </c>
+      <c r="D112" s="23" t="inlineStr">
+        <is>
+          <t>New in report allowance</t>
+        </is>
+      </c>
+      <c r="E112" s="7" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="3" t="n"/>
+      <c r="B113" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.12-4</t>
+        </is>
+      </c>
+      <c r="C113" s="9" t="inlineStr">
+        <is>
+          <t>A mission open to 3 testers leaves Explore after its third report; the builder sees it as inactive.</t>
+        </is>
+      </c>
+      <c r="D113" s="23" t="inlineStr">
+        <is>
+          <t>New in report allowance</t>
+        </is>
+      </c>
+      <c r="E113" s="7" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="3" t="n"/>
+      <c r="B114" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.12-5</t>
+        </is>
+      </c>
+      <c r="C114" s="9" t="inlineStr">
+        <is>
+          <t>Deactivate a live mission that has 1 of 3 reports → the new-mission form shows 2 more available. Reactivate and deactivate again → still correct, never more.</t>
+        </is>
+      </c>
+      <c r="D114" s="23" t="inlineStr">
+        <is>
+          <t>New in report allowance</t>
+        </is>
+      </c>
+      <c r="E114" s="7" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="3" t="n"/>
+      <c r="B115" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.12-6</t>
+        </is>
+      </c>
+      <c r="C115" s="9" t="inlineStr">
+        <is>
+          <t>Create an account, then add the other role → the balance is 3, not 6.</t>
+        </is>
+      </c>
+      <c r="D115" s="23" t="inlineStr">
+        <is>
+          <t>New in report allowance</t>
+        </is>
+      </c>
+      <c r="E115" s="7" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="3" t="n"/>
+      <c r="B116" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.12-7</t>
+        </is>
+      </c>
+      <c r="C116" s="9" t="inlineStr">
+        <is>
+          <t>A Community builder with 2 live missions tries to publish a third → it stays a draft and the page names the 2-mission limit.</t>
+        </is>
+      </c>
+      <c r="D116" s="23" t="inlineStr">
+        <is>
+          <t>New in report allowance</t>
+        </is>
+      </c>
+      <c r="E116" s="7" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="3" t="n"/>
+      <c r="B117" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.12-8</t>
+        </is>
+      </c>
+      <c r="C117" s="9" t="inlineStr">
+        <is>
+          <t>A tester submits on a mission whose builder has 0 reports available → the submission succeeds.</t>
+        </is>
+      </c>
+      <c r="D117" s="23" t="inlineStr">
+        <is>
+          <t>New in report allowance</t>
+        </is>
+      </c>
+      <c r="E117" s="7" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="3" t="n"/>
+      <c r="B118" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.12-9</t>
+        </is>
+      </c>
+      <c r="C118" s="9" t="inlineStr">
+        <is>
+          <t>/admin shows "Uncredited reports" at 0.</t>
+        </is>
+      </c>
+      <c r="D118" s="23" t="inlineStr">
+        <is>
+          <t>New in report allowance</t>
+        </is>
+      </c>
+      <c r="E118" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>

<commit_message>
docs: record the one-report rule and its QA rows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TownHall_Checklist (1).xlsx
+++ b/TownHall_Checklist (1).xlsx
@@ -2683,7 +2683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E108"/>
+  <dimension ref="A1:E111"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4713,6 +4713,51 @@
         </is>
       </c>
       <c r="E108" s="7" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2.12 One report per mission</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="3" t="n"/>
+      <c r="B110" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.12-1</t>
+        </is>
+      </c>
+      <c r="C110" s="9" t="inlineStr">
+        <is>
+          <t>After submitting a report on a mission, reopening it shows "You've tested this mission" instead of the form. Submitting again from a tab opened earlier is refused with "You've already submitted a report for this mission."</t>
+        </is>
+      </c>
+      <c r="D110" s="23" t="inlineStr">
+        <is>
+          <t>New in one report per mission</t>
+        </is>
+      </c>
+      <c r="E110" s="7" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="n"/>
+      <c r="B111" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.12-2</t>
+        </is>
+      </c>
+      <c r="C111" s="9" t="inlineStr">
+        <is>
+          <t>A different tester can still submit on the same mission.</t>
+        </is>
+      </c>
+      <c r="D111" s="23" t="inlineStr">
+        <is>
+          <t>New in one report per mission</t>
+        </is>
+      </c>
+      <c r="E111" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>

<commit_message>
docs: record cohort supply and the payout sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TownHall_Checklist (1).xlsx
+++ b/TownHall_Checklist (1).xlsx
@@ -2683,7 +2683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E121"/>
+  <dimension ref="A1:E128"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4936,6 +4936,127 @@
         </is>
       </c>
       <c r="E121" s="7" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2.14 Cohort payouts</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="3" t="n"/>
+      <c r="B123" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.14-1</t>
+        </is>
+      </c>
+      <c r="C123" s="9" t="inlineStr">
+        <is>
+          <t>In /admin/users, tick "Paid cohort" on a tester → the change appears under "Recent plan and cohort changes" with your name. A user with no tester account shows "No tester account".</t>
+        </is>
+      </c>
+      <c r="D123" s="23" t="inlineStr">
+        <is>
+          <t>New in cohort payouts</t>
+        </is>
+      </c>
+      <c r="E123" s="7" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="3" t="n"/>
+      <c r="B124" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.14-2</t>
+        </is>
+      </c>
+      <c r="C124" s="9" t="inlineStr">
+        <is>
+          <t>Set a builder to Pro, then back to Community → both changes are logged; the builder's settings Plan tab reads Community.</t>
+        </is>
+      </c>
+      <c r="D124" s="23" t="inlineStr">
+        <is>
+          <t>New in cohort payouts</t>
+        </is>
+      </c>
+      <c r="E124" s="7" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="3" t="n"/>
+      <c r="B125" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.14-3</t>
+        </is>
+      </c>
+      <c r="C125" s="9" t="inlineStr">
+        <is>
+          <t>As a cohort tester, Explore and Browse Missions do not list a mission published from earned credit only; opening it by URL shows "This mission isn't paid for cohort testers".</t>
+        </is>
+      </c>
+      <c r="D125" s="23" t="inlineStr">
+        <is>
+          <t>New in cohort payouts</t>
+        </is>
+      </c>
+      <c r="E125" s="7" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="3" t="n"/>
+      <c r="B126" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.14-4</t>
+        </is>
+      </c>
+      <c r="C126" s="9" t="inlineStr">
+        <is>
+          <t>A cohort tester submits on a Pro builder's mission → /admin/payouts for this month shows 1 paid report and ₦1,000.</t>
+        </is>
+      </c>
+      <c r="D126" s="23" t="inlineStr">
+        <is>
+          <t>New in cohort payouts</t>
+        </is>
+      </c>
+      <c r="E126" s="7" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="3" t="n"/>
+      <c r="B127" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.14-5</t>
+        </is>
+      </c>
+      <c r="C127" s="9" t="inlineStr">
+        <is>
+          <t>The month total on /admin/payouts matches the "Month total" row of the downloaded CSV.</t>
+        </is>
+      </c>
+      <c r="D127" s="23" t="inlineStr">
+        <is>
+          <t>New in cohort payouts</t>
+        </is>
+      </c>
+      <c r="E127" s="7" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="3" t="n"/>
+      <c r="B128" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.14-6</t>
+        </is>
+      </c>
+      <c r="C128" s="9" t="inlineStr">
+        <is>
+          <t>Take a tester out of the cohort → last month's payout sheet is unchanged.</t>
+        </is>
+      </c>
+      <c r="D128" s="23" t="inlineStr">
+        <is>
+          <t>New in cohort payouts</t>
+        </is>
+      </c>
+      <c r="E128" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>

<commit_message>
Document rate limiting: CLAUDE.md, .env.example, QA rows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TownHall_Checklist (1).xlsx
+++ b/TownHall_Checklist (1).xlsx
@@ -2683,7 +2683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E132"/>
+  <dimension ref="A1:E138"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2875,7 +2875,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="19.5" customHeight="1">
       <c r="A11" s="39" t="inlineStr">
         <is>
@@ -3014,7 +3013,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="19.5" customHeight="1">
       <c r="A18" s="39" t="inlineStr">
         <is>
@@ -3184,7 +3182,6 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
     <row r="26" ht="19.5" customHeight="1">
       <c r="A26" s="39" t="inlineStr">
         <is>
@@ -3346,7 +3343,6 @@
         </is>
       </c>
     </row>
-    <row r="33"/>
     <row r="34" ht="19.5" customHeight="1">
       <c r="A34" s="39" t="inlineStr">
         <is>
@@ -3435,7 +3431,6 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
     <row r="39" ht="19.5" customHeight="1">
       <c r="A39" s="39" t="inlineStr">
         <is>
@@ -3520,7 +3515,6 @@
         </is>
       </c>
     </row>
-    <row r="43"/>
     <row r="44" ht="19.5" customHeight="1">
       <c r="A44" s="39" t="inlineStr">
         <is>
@@ -3767,7 +3761,6 @@
         </is>
       </c>
     </row>
-    <row r="54"/>
     <row r="55" ht="19.5" customHeight="1">
       <c r="A55" s="39" t="inlineStr">
         <is>
@@ -3883,7 +3876,6 @@
         </is>
       </c>
     </row>
-    <row r="60"/>
     <row r="61">
       <c r="A61" s="39" t="n"/>
       <c r="C61" t="inlineStr">
@@ -4177,7 +4169,6 @@
       </c>
       <c r="E76" s="7" t="n"/>
     </row>
-    <row r="77"/>
     <row r="78">
       <c r="A78" s="39" t="n"/>
       <c r="C78" t="inlineStr">
@@ -4471,7 +4462,6 @@
       </c>
       <c r="E93" s="7" t="inlineStr"/>
     </row>
-    <row r="94"/>
     <row r="95">
       <c r="A95" s="39" t="n"/>
       <c r="C95" t="inlineStr">
@@ -4727,7 +4717,6 @@
       </c>
       <c r="E108" s="7" t="n"/>
     </row>
-    <row r="109"/>
     <row r="110">
       <c r="A110" s="39" t="n"/>
       <c r="C110" t="inlineStr">
@@ -5120,6 +5109,109 @@
         </is>
       </c>
       <c r="E132" s="7" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="39" t="n"/>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2.16 Rate limiting</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="3" t="n"/>
+      <c r="B134" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.16-1</t>
+        </is>
+      </c>
+      <c r="C134" s="9" t="inlineStr">
+        <is>
+          <t>Enter a wrong password eleven times in a row on one address → "Too many attempts. Try again in N minutes." Do the same on an address with no account → the same message, just as fast. The message never states how many attempts are allowed.</t>
+        </is>
+      </c>
+      <c r="D134" s="23" t="inlineStr">
+        <is>
+          <t>New in rate limiting</t>
+        </is>
+      </c>
+      <c r="E134" s="7" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="3" t="n"/>
+      <c r="B135" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.16-2</t>
+        </is>
+      </c>
+      <c r="C135" s="9" t="inlineStr">
+        <is>
+          <t>The limited sign-in message renders in danger-ink on both light and dark themes, and wraps cleanly at 360px width.</t>
+        </is>
+      </c>
+      <c r="D135" s="23" t="inlineStr">
+        <is>
+          <t>New in rate limiting</t>
+        </is>
+      </c>
+      <c r="E135" s="7" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="3" t="n"/>
+      <c r="B136" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.16-3</t>
+        </is>
+      </c>
+      <c r="C136" s="9" t="inlineStr">
+        <is>
+          <t>As a tester, submit reports on eleven different missions within an hour → the eleventh is refused with "Try again in N minutes" and no screenshots are uploaded.</t>
+        </is>
+      </c>
+      <c r="D136" s="23" t="inlineStr">
+        <is>
+          <t>New in rate limiting</t>
+        </is>
+      </c>
+      <c r="E136" s="7" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="3" t="n"/>
+      <c r="B137" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.16-4</t>
+        </is>
+      </c>
+      <c r="C137" s="9" t="inlineStr">
+        <is>
+          <t>With rate_limit_hit unavailable on staging (execute revoked from service_role): sign-in still works and the server log shows "[rate-limit] store unavailable, degrading"; a test submission is refused with "Try again in a minute".</t>
+        </is>
+      </c>
+      <c r="D137" s="23" t="inlineStr">
+        <is>
+          <t>New in rate limiting</t>
+        </is>
+      </c>
+      <c r="E137" s="7" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="3" t="n"/>
+      <c r="B138" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.16-5</t>
+        </is>
+      </c>
+      <c r="C138" s="9" t="inlineStr">
+        <is>
+          <t>Set RATE_LIMIT_DISABLED=true and redeploy → the eleven wrong passwords are all answered "That email and password do not match."; every check logs "[rate-limit] DISABLED". Unset it and redeploy → limits are back.</t>
+        </is>
+      </c>
+      <c r="D138" s="23" t="inlineStr">
+        <is>
+          <t>New in rate limiting</t>
+        </is>
+      </c>
+      <c r="E138" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>

<commit_message>
Update QA checklist progress
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TownHall_Checklist (1).xlsx
+++ b/TownHall_Checklist (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\townhall\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D09BEAA6-DC51-408E-85BD-07EFC58397B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01605A86-E2AE-406E-925A-109B65E044AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="853" uniqueCount="487">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="877" uniqueCount="487">
   <si>
     <t>TownHall — 1 · Engineer Tests</t>
   </si>
@@ -2045,6 +2045,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFFE6E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFE2EFDA"/>
         </patternFill>
       </fill>
@@ -2052,6 +2059,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFFE6E6"/>
         </patternFill>
       </fill>
@@ -2059,6 +2073,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFE2EFDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFFF2CC"/>
         </patternFill>
       </fill>
@@ -2129,6 +2150,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFFE6E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFE2EFDA"/>
         </patternFill>
       </fill>
@@ -2136,6 +2164,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFFE6E6"/>
         </patternFill>
       </fill>
@@ -2143,6 +2178,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFE2EFDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFFF2CC"/>
         </patternFill>
       </fill>
@@ -2164,6 +2206,20 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFE6E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFE2EFDA"/>
         </patternFill>
       </fill>
@@ -2185,6 +2241,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFE2EFDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFFF2CC"/>
         </patternFill>
       </fill>
@@ -2311,6 +2374,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFFE6E6"/>
         </patternFill>
       </fill>
@@ -2319,76 +2389,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFE2EFDA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFE6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE2EFDA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFE6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE2EFDA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE2EFDA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFE6E6"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3641,11 +3641,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A20:E24">
-    <cfRule type="expression" dxfId="59" priority="36">
+    <cfRule type="expression" dxfId="59" priority="35">
+      <formula>$E20="Done"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="58" priority="36">
       <formula>$E20="Blocked"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="58" priority="35">
-      <formula>$E20="Done"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="57" priority="37">
       <formula>$E20="In Progress"</formula>
@@ -3663,25 +3663,25 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A35:E40">
-    <cfRule type="expression" dxfId="53" priority="70">
+    <cfRule type="expression" dxfId="53" priority="68">
+      <formula>$E35="Done"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="52" priority="69">
+      <formula>$E35="Blocked"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="51" priority="70">
       <formula>$E35="In Progress"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="52" priority="68">
-      <formula>$E35="Done"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="51" priority="69">
-      <formula>$E35="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A43:E51">
-    <cfRule type="expression" dxfId="50" priority="88">
+    <cfRule type="expression" dxfId="50" priority="86">
+      <formula>$E43="Done"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="49" priority="87">
+      <formula>$E43="Blocked"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="48" priority="88">
       <formula>$E43="In Progress"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="49" priority="86">
-      <formula>$E43="Done"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="48" priority="87">
-      <formula>$E43="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A54:E56">
@@ -3752,14 +3752,14 @@
     <row r="2" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="53" t="str">
         <f>IFERROR(COUNTIF(E4:E2000,"Done")&amp;" / "&amp;COUNTA(B4:B2000)&amp;" items completed","0 / 0 items completed")</f>
-        <v>64 / 108 items completed</v>
+        <v>86 / 108 items completed</v>
       </c>
       <c r="B2" s="51"/>
       <c r="C2" s="51"/>
       <c r="D2" s="51"/>
       <c r="E2" s="11">
         <f>IFERROR(COUNTIF(E4:E2000,"Done")/COUNTA(B4:B2000),0)</f>
-        <v>0.59259259259259256</v>
+        <v>0.79629629629629628</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -5011,7 +5011,9 @@
       <c r="D96" s="23" t="s">
         <v>324</v>
       </c>
-      <c r="E96" s="7"/>
+      <c r="E96" s="7" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="97" spans="1:5" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A97" s="3"/>
@@ -5024,7 +5026,9 @@
       <c r="D97" s="23" t="s">
         <v>324</v>
       </c>
-      <c r="E97" s="7"/>
+      <c r="E97" s="7" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="98" spans="1:5" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A98" s="3"/>
@@ -5037,7 +5041,9 @@
       <c r="D98" s="23" t="s">
         <v>324</v>
       </c>
-      <c r="E98" s="7"/>
+      <c r="E98" s="7" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="99" spans="1:5" ht="34.200000000000003" x14ac:dyDescent="0.3">
       <c r="A99" s="3"/>
@@ -5050,7 +5056,9 @@
       <c r="D99" s="23" t="s">
         <v>324</v>
       </c>
-      <c r="E99" s="7"/>
+      <c r="E99" s="7" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="100" spans="1:5" ht="34.200000000000003" x14ac:dyDescent="0.3">
       <c r="A100" s="3"/>
@@ -5063,7 +5071,9 @@
       <c r="D100" s="23" t="s">
         <v>324</v>
       </c>
-      <c r="E100" s="7"/>
+      <c r="E100" s="7" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="101" spans="1:5" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A101" s="3"/>
@@ -5076,7 +5086,9 @@
       <c r="D101" s="23" t="s">
         <v>324</v>
       </c>
-      <c r="E101" s="7"/>
+      <c r="E101" s="7" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="102" spans="1:5" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A102" s="3"/>
@@ -5089,7 +5101,9 @@
       <c r="D102" s="23" t="s">
         <v>324</v>
       </c>
-      <c r="E102" s="7"/>
+      <c r="E102" s="7" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="103" spans="1:5" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A103" s="3"/>
@@ -5102,7 +5116,9 @@
       <c r="D103" s="23" t="s">
         <v>324</v>
       </c>
-      <c r="E103" s="7"/>
+      <c r="E103" s="7" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="104" spans="1:5" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A104" s="3"/>
@@ -5115,7 +5131,9 @@
       <c r="D104" s="23" t="s">
         <v>324</v>
       </c>
-      <c r="E104" s="7"/>
+      <c r="E104" s="7" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="105" spans="1:5" ht="34.200000000000003" x14ac:dyDescent="0.3">
       <c r="A105" s="3"/>
@@ -5128,7 +5146,9 @@
       <c r="D105" s="23" t="s">
         <v>324</v>
       </c>
-      <c r="E105" s="7"/>
+      <c r="E105" s="7" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="106" spans="1:5" ht="34.200000000000003" x14ac:dyDescent="0.3">
       <c r="A106" s="3"/>
@@ -5141,7 +5161,9 @@
       <c r="D106" s="23" t="s">
         <v>324</v>
       </c>
-      <c r="E106" s="7"/>
+      <c r="E106" s="7" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="107" spans="1:5" ht="34.200000000000003" x14ac:dyDescent="0.3">
       <c r="A107" s="3"/>
@@ -5154,7 +5176,9 @@
       <c r="D107" s="23" t="s">
         <v>324</v>
       </c>
-      <c r="E107" s="7"/>
+      <c r="E107" s="7" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="108" spans="1:5" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A108" s="3"/>
@@ -5167,7 +5191,9 @@
       <c r="D108" s="23" t="s">
         <v>324</v>
       </c>
-      <c r="E108" s="7"/>
+      <c r="E108" s="7" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A110" s="36"/>
@@ -5218,7 +5244,9 @@
       <c r="D114" s="23" t="s">
         <v>358</v>
       </c>
-      <c r="E114" s="7"/>
+      <c r="E114" s="7" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="115" spans="1:5" ht="34.200000000000003" x14ac:dyDescent="0.3">
       <c r="A115" s="3"/>
@@ -5231,7 +5259,9 @@
       <c r="D115" s="23" t="s">
         <v>358</v>
       </c>
-      <c r="E115" s="7"/>
+      <c r="E115" s="7" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="116" spans="1:5" ht="34.200000000000003" x14ac:dyDescent="0.3">
       <c r="A116" s="3"/>
@@ -5244,7 +5274,9 @@
       <c r="D116" s="23" t="s">
         <v>358</v>
       </c>
-      <c r="E116" s="7"/>
+      <c r="E116" s="7" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="117" spans="1:5" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A117" s="3"/>
@@ -5270,7 +5302,9 @@
       <c r="D118" s="23" t="s">
         <v>358</v>
       </c>
-      <c r="E118" s="7"/>
+      <c r="E118" s="7" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="119" spans="1:5" ht="15" x14ac:dyDescent="0.3">
       <c r="A119" s="3"/>
@@ -5283,7 +5317,9 @@
       <c r="D119" s="23" t="s">
         <v>358</v>
       </c>
-      <c r="E119" s="7"/>
+      <c r="E119" s="7" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="120" spans="1:5" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A120" s="3"/>
@@ -5296,7 +5332,9 @@
       <c r="D120" s="23" t="s">
         <v>358</v>
       </c>
-      <c r="E120" s="7"/>
+      <c r="E120" s="7" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="121" spans="1:5" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A121" s="3"/>
@@ -5309,7 +5347,9 @@
       <c r="D121" s="23" t="s">
         <v>358</v>
       </c>
-      <c r="E121" s="7"/>
+      <c r="E121" s="7" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="122" spans="1:5" ht="15" x14ac:dyDescent="0.3">
       <c r="A122" s="3"/>
@@ -5341,7 +5381,9 @@
       <c r="D124" s="23" t="s">
         <v>378</v>
       </c>
-      <c r="E124" s="7"/>
+      <c r="E124" s="7" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="125" spans="1:5" ht="15" x14ac:dyDescent="0.3">
       <c r="A125" s="3"/>
@@ -5354,7 +5396,9 @@
       <c r="D125" s="23" t="s">
         <v>378</v>
       </c>
-      <c r="E125" s="7"/>
+      <c r="E125" s="7" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A126" s="36"/>
@@ -5513,16 +5557,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A55:E55"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A11:E11"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A44:E44"/>
     <mergeCell ref="A18:E18"/>
     <mergeCell ref="A39:E39"/>
     <mergeCell ref="A34:E34"/>
-    <mergeCell ref="A55:E55"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A26:E26"/>
-    <mergeCell ref="A11:E11"/>
   </mergeCells>
   <conditionalFormatting sqref="A5:E9">
     <cfRule type="expression" dxfId="38" priority="2">
@@ -5558,14 +5602,14 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A27:E32">
-    <cfRule type="expression" dxfId="29" priority="51">
+    <cfRule type="expression" dxfId="29" priority="50">
+      <formula>$E27="Done"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="28" priority="51">
       <formula>$E27="Blocked"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="28" priority="52">
+    <cfRule type="expression" dxfId="27" priority="52">
       <formula>$E27="In Progress"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="27" priority="50">
-      <formula>$E27="Done"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A35:E37">
@@ -5580,11 +5624,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A40:E42">
-    <cfRule type="expression" dxfId="23" priority="78">
+    <cfRule type="expression" dxfId="23" priority="77">
+      <formula>$E40="Done"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="22" priority="78">
       <formula>$E40="Blocked"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="22" priority="77">
-      <formula>$E40="Done"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="21" priority="79">
       <formula>$E40="In Progress"</formula>
@@ -5647,14 +5691,14 @@
     <row r="2" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="53" t="str">
         <f>IFERROR(COUNTIF(E4:E2000,"Done")&amp;" / "&amp;COUNTA(B4:B2000)&amp;" items completed","0 / 0 items completed")</f>
-        <v>12 / 19 items completed</v>
+        <v>14 / 19 items completed</v>
       </c>
       <c r="B2" s="51"/>
       <c r="C2" s="51"/>
       <c r="D2" s="51"/>
       <c r="E2" s="13">
         <f>IFERROR(COUNTIF(E4:E2000,"Done")/COUNTA(B4:B2000),0)</f>
-        <v>0.63157894736842102</v>
+        <v>0.73684210526315785</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -5980,8 +6024,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="105.6" x14ac:dyDescent="0.3">
-      <c r="A27" s="37" t="s">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C27" s="37" t="s">
         <v>447</v>
       </c>
     </row>
@@ -5996,7 +6040,9 @@
       <c r="D28" s="34" t="s">
         <v>260</v>
       </c>
-      <c r="E28" s="7"/>
+      <c r="E28" s="7" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="29" spans="1:5" ht="15" x14ac:dyDescent="0.3">
       <c r="A29" s="3"/>
@@ -6009,7 +6055,9 @@
       <c r="D29" s="34" t="s">
         <v>260</v>
       </c>
-      <c r="E29" s="7"/>
+      <c r="E29" s="7" t="s">
+        <v>159</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -6031,11 +6079,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A15:E19">
-    <cfRule type="expression" dxfId="11" priority="27">
+    <cfRule type="expression" dxfId="11" priority="26">
+      <formula>$E15="Done"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="10" priority="27">
       <formula>$E15="Blocked"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="10" priority="26">
-      <formula>$E15="Done"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="9" priority="28">
       <formula>$E15="In Progress"</formula>

</xml_diff>

<commit_message>
Update the 2.17 checklist rows for the new export
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TownHall_Checklist (1).xlsx
+++ b/TownHall_Checklist (1).xlsx
@@ -307,7 +307,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -412,12 +412,6 @@
     <xf numFmtId="0" fontId="19" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -454,6 +448,13 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -464,11 +465,11 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1208,22 +1209,22 @@
   <dimension ref="A1:E66"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
-    <col width="5" customWidth="1" style="51" min="1" max="1"/>
-    <col width="12" customWidth="1" style="51" min="2" max="2"/>
-    <col width="58" customWidth="1" style="51" min="3" max="3"/>
-    <col width="36" customWidth="1" style="51" min="4" max="4"/>
-    <col width="14" customWidth="1" style="51" min="5" max="5"/>
+    <col width="5" customWidth="1" style="52" min="1" max="1"/>
+    <col width="12" customWidth="1" style="52" min="2" max="2"/>
+    <col width="58" customWidth="1" style="52" min="3" max="3"/>
+    <col width="36" customWidth="1" style="52" min="4" max="4"/>
+    <col width="14" customWidth="1" style="52" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" s="51">
-      <c r="A1" s="52" t="inlineStr">
+    <row r="1" ht="31.5" customHeight="1" s="52">
+      <c r="A1" s="53" t="inlineStr">
         <is>
           <t>TownHall — 1 · Engineer Tests</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="19.5" customHeight="1" s="51">
-      <c r="A2" s="53">
+    <row r="2" ht="19.5" customHeight="1" s="52">
+      <c r="A2" s="54">
         <f>IFERROR(COUNTIF(E4:E2000,"Done")&amp;" / "&amp;COUNTA(B4:B2000)&amp;" items completed","0 / 0 items completed")</f>
         <v/>
       </c>
@@ -1232,7 +1233,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="21.75" customHeight="1" s="51">
+    <row r="3" ht="21.75" customHeight="1" s="52">
       <c r="A3" s="2" t="n"/>
       <c r="B3" s="2" t="inlineStr">
         <is>
@@ -1255,14 +1256,14 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="19.5" customHeight="1" s="51">
-      <c r="A4" s="50" t="inlineStr">
+    <row r="4" ht="19.5" customHeight="1" s="52">
+      <c r="A4" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">  1.1 Authentication — actions/auth.ts</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="21.75" customHeight="1" s="51">
+    <row r="5" ht="21.75" customHeight="1" s="52">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -1289,7 +1290,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1" s="51">
+    <row r="6" ht="30" customHeight="1" s="52">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -1316,7 +1317,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="30" customHeight="1" s="51">
+    <row r="7" ht="30" customHeight="1" s="52">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -1343,7 +1344,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="21.75" customHeight="1" s="51">
+    <row r="8" ht="21.75" customHeight="1" s="52">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -1370,7 +1371,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="21.75" customHeight="1" s="51">
+    <row r="9" ht="21.75" customHeight="1" s="52">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -1397,7 +1398,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="21.75" customHeight="1" s="51">
+    <row r="10" ht="21.75" customHeight="1" s="52">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -1424,7 +1425,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="21.75" customHeight="1" s="51">
+    <row r="11" ht="21.75" customHeight="1" s="52">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -1451,14 +1452,14 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="19.5" customHeight="1" s="51">
-      <c r="A13" s="50" t="inlineStr">
+    <row r="13" ht="19.5" customHeight="1" s="52">
+      <c r="A13" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">  1.2 Middleware — middleware.ts</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="21.75" customHeight="1" s="51">
+    <row r="14" ht="21.75" customHeight="1" s="52">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -1485,7 +1486,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="21.75" customHeight="1" s="51">
+    <row r="15" ht="21.75" customHeight="1" s="52">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -1512,7 +1513,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="21.75" customHeight="1" s="51">
+    <row r="16" ht="21.75" customHeight="1" s="52">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -1539,7 +1540,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="21.75" customHeight="1" s="51">
+    <row r="17" ht="21.75" customHeight="1" s="52">
       <c r="A17" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -1566,14 +1567,14 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="19.5" customHeight="1" s="51">
-      <c r="A19" s="50" t="inlineStr">
+    <row r="19" ht="19.5" customHeight="1" s="52">
+      <c r="A19" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">  1.3 Projects — actions/project.ts</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="21.75" customHeight="1" s="51">
+    <row r="20" ht="21.75" customHeight="1" s="52">
       <c r="A20" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -1600,7 +1601,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="21.75" customHeight="1" s="51">
+    <row r="21" ht="21.75" customHeight="1" s="52">
       <c r="A21" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -1627,7 +1628,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="21.75" customHeight="1" s="51">
+    <row r="22" ht="21.75" customHeight="1" s="52">
       <c r="A22" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -1654,7 +1655,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="21.75" customHeight="1" s="51">
+    <row r="23" ht="21.75" customHeight="1" s="52">
       <c r="A23" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -1681,7 +1682,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="21.75" customHeight="1" s="51">
+    <row r="24" ht="21.75" customHeight="1" s="52">
       <c r="A24" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -1708,14 +1709,14 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="19.5" customHeight="1" s="51">
-      <c r="A26" s="50" t="inlineStr">
+    <row r="26" ht="19.5" customHeight="1" s="52">
+      <c r="A26" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">  1.4 Missions — actions/missions.ts</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="21.75" customHeight="1" s="51">
+    <row r="27" ht="21.75" customHeight="1" s="52">
       <c r="A27" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -1742,7 +1743,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="21.75" customHeight="1" s="51">
+    <row r="28" ht="21.75" customHeight="1" s="52">
       <c r="A28" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -1769,7 +1770,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="21.75" customHeight="1" s="51">
+    <row r="29" ht="21.75" customHeight="1" s="52">
       <c r="A29" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -1796,7 +1797,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="21.75" customHeight="1" s="51">
+    <row r="30" ht="21.75" customHeight="1" s="52">
       <c r="A30" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -1823,7 +1824,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="21.75" customHeight="1" s="51">
+    <row r="31" ht="21.75" customHeight="1" s="52">
       <c r="A31" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -1850,7 +1851,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="21.75" customHeight="1" s="51">
+    <row r="32" ht="21.75" customHeight="1" s="52">
       <c r="A32" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -1877,14 +1878,14 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="19.5" customHeight="1" s="51">
-      <c r="A34" s="50" t="inlineStr">
+    <row r="34" ht="19.5" customHeight="1" s="52">
+      <c r="A34" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">  1.5 Submissions / AI — actions/submissions.ts, lib/ai</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="21.75" customHeight="1" s="51">
+    <row r="35" ht="21.75" customHeight="1" s="52">
       <c r="A35" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -1911,7 +1912,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="21.75" customHeight="1" s="51">
+    <row r="36" ht="21.75" customHeight="1" s="52">
       <c r="A36" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -1938,7 +1939,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="21.75" customHeight="1" s="51">
+    <row r="37" ht="21.75" customHeight="1" s="52">
       <c r="A37" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -1965,7 +1966,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="21.75" customHeight="1" s="51">
+    <row r="38" ht="21.75" customHeight="1" s="52">
       <c r="A38" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -1992,7 +1993,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="21.75" customHeight="1" s="51">
+    <row r="39" ht="21.75" customHeight="1" s="52">
       <c r="A39" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -2019,7 +2020,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="21.75" customHeight="1" s="51">
+    <row r="40" ht="21.75" customHeight="1" s="52">
       <c r="A40" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -2046,14 +2047,14 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="19.5" customHeight="1" s="51">
-      <c r="A42" s="50" t="inlineStr">
+    <row r="42" ht="19.5" customHeight="1" s="52">
+      <c r="A42" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">  1.6 Admin Broadcast — actions/admin/broadcast.ts</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="21.75" customHeight="1" s="51">
+    <row r="43" ht="21.75" customHeight="1" s="52">
       <c r="A43" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -2080,7 +2081,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="21.75" customHeight="1" s="51">
+    <row r="44" ht="21.75" customHeight="1" s="52">
       <c r="A44" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -2107,7 +2108,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="21.75" customHeight="1" s="51">
+    <row r="45" ht="21.75" customHeight="1" s="52">
       <c r="A45" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -2134,7 +2135,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="21.75" customHeight="1" s="51">
+    <row r="46" ht="21.75" customHeight="1" s="52">
       <c r="A46" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -2161,7 +2162,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="21.75" customHeight="1" s="51">
+    <row r="47" ht="21.75" customHeight="1" s="52">
       <c r="A47" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -2188,7 +2189,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="21.75" customHeight="1" s="51">
+    <row r="48" ht="21.75" customHeight="1" s="52">
       <c r="A48" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -2215,7 +2216,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="21.75" customHeight="1" s="51">
+    <row r="49" ht="21.75" customHeight="1" s="52">
       <c r="A49" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -2242,7 +2243,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="21.75" customHeight="1" s="51">
+    <row r="50" ht="21.75" customHeight="1" s="52">
       <c r="A50" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -2269,7 +2270,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="21.75" customHeight="1" s="51">
+    <row r="51" ht="21.75" customHeight="1" s="52">
       <c r="A51" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -2296,14 +2297,14 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="19.5" customHeight="1" s="51">
-      <c r="A53" s="50" t="inlineStr">
+    <row r="53" ht="19.5" customHeight="1" s="52">
+      <c r="A53" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">  1.7 Email &amp; Notifications — emails/, lib/mail.ts</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="21.75" customHeight="1" s="51">
+    <row r="54" ht="21.75" customHeight="1" s="52">
       <c r="A54" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -2330,7 +2331,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="21.75" customHeight="1" s="51">
+    <row r="55" ht="21.75" customHeight="1" s="52">
       <c r="A55" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -2357,7 +2358,7 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="21.75" customHeight="1" s="51">
+    <row r="56" ht="21.75" customHeight="1" s="52">
       <c r="A56" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -2384,14 +2385,14 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="19.5" customHeight="1" s="51">
-      <c r="A58" s="50" t="inlineStr">
+    <row r="58" ht="19.5" customHeight="1" s="52">
+      <c r="A58" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">  1.8 Webhook — app/api/webhooks/submission</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="21.75" customHeight="1" s="51">
+    <row r="59" ht="21.75" customHeight="1" s="52">
       <c r="A59" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -2418,7 +2419,7 @@
         </is>
       </c>
     </row>
-    <row r="60" ht="21.75" customHeight="1" s="51">
+    <row r="60" ht="21.75" customHeight="1" s="52">
       <c r="A60" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -2445,7 +2446,7 @@
         </is>
       </c>
     </row>
-    <row r="61" ht="21.75" customHeight="1" s="51">
+    <row r="61" ht="21.75" customHeight="1" s="52">
       <c r="A61" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -2472,14 +2473,14 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="19.5" customHeight="1" s="51">
-      <c r="A63" s="50" t="inlineStr">
+    <row r="63" ht="19.5" customHeight="1" s="52">
+      <c r="A63" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">  1.9 Type &amp; Lint Gates</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="21.75" customHeight="1" s="51">
+    <row r="64" ht="21.75" customHeight="1" s="52">
       <c r="A64" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -2506,7 +2507,7 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="21.75" customHeight="1" s="51">
+    <row r="65" ht="21.75" customHeight="1" s="52">
       <c r="A65" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -2533,7 +2534,7 @@
         </is>
       </c>
     </row>
-    <row r="66" ht="21.75" customHeight="1" s="51">
+    <row r="66" ht="21.75" customHeight="1" s="52">
       <c r="A66" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -2570,8 +2571,8 @@
     <mergeCell ref="A19:E19"/>
     <mergeCell ref="A63:E63"/>
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A13:E13"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A13:E13"/>
     <mergeCell ref="A58:E58"/>
   </mergeCells>
   <conditionalFormatting sqref="A5:E11">
@@ -2690,25 +2691,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E146"/>
+  <dimension ref="A1:E147"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
-    <col width="5" customWidth="1" style="51" min="1" max="1"/>
-    <col width="12" customWidth="1" style="51" min="2" max="2"/>
-    <col width="58" customWidth="1" style="51" min="3" max="3"/>
-    <col width="36" customWidth="1" style="51" min="4" max="4"/>
-    <col width="14" customWidth="1" style="51" min="5" max="5"/>
+    <col width="5" customWidth="1" style="52" min="1" max="1"/>
+    <col width="12" customWidth="1" style="52" min="2" max="2"/>
+    <col width="58" customWidth="1" style="52" min="3" max="3"/>
+    <col width="36" customWidth="1" style="52" min="4" max="4"/>
+    <col width="14" customWidth="1" style="52" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" s="51">
+    <row r="1" ht="31.5" customHeight="1" s="52">
       <c r="A1" s="55" t="inlineStr">
         <is>
           <t>TownHall — 2 · QA Tester</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="19.5" customHeight="1" s="51">
-      <c r="A2" s="53">
+    <row r="2" ht="19.5" customHeight="1" s="52">
+      <c r="A2" s="54">
         <f>IFERROR(COUNTIF(E4:E2000,"Done")&amp;" / "&amp;COUNTA(B4:B2000)&amp;" items completed","0 / 0 items completed")</f>
         <v/>
       </c>
@@ -2717,7 +2718,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="21.75" customHeight="1" s="51">
+    <row r="3" ht="21.75" customHeight="1" s="52">
       <c r="A3" s="12" t="n"/>
       <c r="B3" s="12" t="inlineStr">
         <is>
@@ -2740,14 +2741,14 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="19.5" customHeight="1" s="51">
-      <c r="A4" s="54" t="inlineStr">
+    <row r="4" ht="19.5" customHeight="1" s="52">
+      <c r="A4" s="56" t="inlineStr">
         <is>
           <t xml:space="preserve">  2.1 Onboarding &amp; Auth</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1" s="51">
+    <row r="5" ht="30" customHeight="1" s="52">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -2774,7 +2775,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1" s="51">
+    <row r="6" ht="30" customHeight="1" s="52">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -2801,7 +2802,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="21.75" customHeight="1" s="51">
+    <row r="7" ht="21.75" customHeight="1" s="52">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -2828,7 +2829,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="30" customHeight="1" s="51">
+    <row r="8" ht="30" customHeight="1" s="52">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -2882,14 +2883,14 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="19.5" customHeight="1" s="51">
-      <c r="A11" s="54" t="inlineStr">
+    <row r="11" ht="19.5" customHeight="1" s="52">
+      <c r="A11" s="56" t="inlineStr">
         <is>
           <t xml:space="preserve">  2.2 Developer Flow — Submit a Project</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="21.75" customHeight="1" s="51">
+    <row r="12" ht="21.75" customHeight="1" s="52">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -2916,7 +2917,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="30" customHeight="1" s="51">
+    <row r="13" ht="30" customHeight="1" s="52">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -2939,7 +2940,7 @@
       </c>
       <c r="E13" s="7" t="n"/>
     </row>
-    <row r="14" ht="21.75" customHeight="1" s="51">
+    <row r="14" ht="21.75" customHeight="1" s="52">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -2966,7 +2967,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="30" customHeight="1" s="51">
+    <row r="15" ht="30" customHeight="1" s="52">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -2993,7 +2994,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="21.75" customHeight="1" s="51">
+    <row r="16" ht="21.75" customHeight="1" s="52">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -3020,14 +3021,14 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="19.5" customHeight="1" s="51">
-      <c r="A18" s="54" t="inlineStr">
+    <row r="18" ht="19.5" customHeight="1" s="52">
+      <c r="A18" s="56" t="inlineStr">
         <is>
           <t xml:space="preserve">  2.3 Developer Flow — Create &amp; Manage Missions</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="30" customHeight="1" s="51">
+    <row r="19" ht="30" customHeight="1" s="52">
       <c r="A19" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -3054,7 +3055,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="21.75" customHeight="1" s="51">
+    <row r="20" ht="21.75" customHeight="1" s="52">
       <c r="A20" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -3081,7 +3082,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="21.75" customHeight="1" s="51">
+    <row r="21" ht="21.75" customHeight="1" s="52">
       <c r="A21" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -3108,7 +3109,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="30" customHeight="1" s="51">
+    <row r="22" ht="30" customHeight="1" s="52">
       <c r="A22" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -3162,7 +3163,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="21.75" customHeight="1" s="51">
+    <row r="24" ht="21.75" customHeight="1" s="52">
       <c r="A24" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -3189,14 +3190,14 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="19.5" customHeight="1" s="51">
-      <c r="A26" s="54" t="inlineStr">
+    <row r="26" ht="19.5" customHeight="1" s="52">
+      <c r="A26" s="56" t="inlineStr">
         <is>
           <t xml:space="preserve">  2.4 Tester Flow — Discover &amp; Test</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="21.75" customHeight="1" s="51">
+    <row r="27" ht="21.75" customHeight="1" s="52">
       <c r="A27" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -3223,7 +3224,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="30" customHeight="1" s="51">
+    <row r="28" ht="30" customHeight="1" s="52">
       <c r="A28" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -3250,7 +3251,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="30" customHeight="1" s="51">
+    <row r="29" ht="30" customHeight="1" s="52">
       <c r="A29" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -3273,7 +3274,7 @@
       </c>
       <c r="E29" s="7" t="n"/>
     </row>
-    <row r="30" ht="30" customHeight="1" s="51">
+    <row r="30" ht="30" customHeight="1" s="52">
       <c r="A30" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -3296,7 +3297,7 @@
       </c>
       <c r="E30" s="7" t="n"/>
     </row>
-    <row r="31" ht="30" customHeight="1" s="51">
+    <row r="31" ht="30" customHeight="1" s="52">
       <c r="A31" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -3323,7 +3324,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="30" customHeight="1" s="51">
+    <row r="32" ht="30" customHeight="1" s="52">
       <c r="A32" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -3350,14 +3351,14 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="19.5" customHeight="1" s="51">
-      <c r="A34" s="54" t="inlineStr">
+    <row r="34" ht="19.5" customHeight="1" s="52">
+      <c r="A34" s="56" t="inlineStr">
         <is>
           <t xml:space="preserve">  2.5 AI Analysis</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="30" customHeight="1" s="51">
+    <row r="35" ht="30" customHeight="1" s="52">
       <c r="A35" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -3384,7 +3385,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="21.75" customHeight="1" s="51">
+    <row r="36" ht="21.75" customHeight="1" s="52">
       <c r="A36" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -3412,40 +3413,40 @@
       </c>
     </row>
     <row r="37" ht="30" customFormat="1" customHeight="1" s="22">
-      <c r="A37" s="45" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B37" s="46" t="inlineStr">
+      <c r="A37" s="43" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B37" s="44" t="inlineStr">
         <is>
           <t>QA-2.5-3</t>
         </is>
       </c>
-      <c r="C37" s="47" t="inlineStr">
+      <c r="C37" s="45" t="inlineStr">
         <is>
           <t>Simulate Gemini outage → submission still saves; empty summary, sentiment defaults to NEUTRAL</t>
         </is>
       </c>
-      <c r="D37" s="48" t="inlineStr">
+      <c r="D37" s="46" t="inlineStr">
         <is>
           <t>No issues</t>
         </is>
       </c>
-      <c r="E37" s="49" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="19.5" customHeight="1" s="51">
-      <c r="A39" s="54" t="inlineStr">
+      <c r="E37" s="47" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="19.5" customHeight="1" s="52">
+      <c r="A39" s="56" t="inlineStr">
         <is>
           <t xml:space="preserve">  2.6 Notifications &amp; Email</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="30" customHeight="1" s="51">
+    <row r="40" ht="30" customHeight="1" s="52">
       <c r="A40" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -3472,7 +3473,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="30" customHeight="1" s="51">
+    <row r="41" ht="30" customHeight="1" s="52">
       <c r="A41" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -3499,7 +3500,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="30" customHeight="1" s="51">
+    <row r="42" ht="30" customHeight="1" s="52">
       <c r="A42" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -3522,14 +3523,14 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="19.5" customHeight="1" s="51">
-      <c r="A44" s="54" t="inlineStr">
+    <row r="44" ht="19.5" customHeight="1" s="52">
+      <c r="A44" s="56" t="inlineStr">
         <is>
           <t xml:space="preserve">  2.7 Admin Console — /admin</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="21.75" customHeight="1" s="51">
+    <row r="45" ht="21.75" customHeight="1" s="52">
       <c r="A45" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -3556,7 +3557,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="30" customHeight="1" s="51">
+    <row r="46" ht="30" customHeight="1" s="52">
       <c r="A46" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -3583,7 +3584,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="30" customHeight="1" s="51">
+    <row r="47" ht="30" customHeight="1" s="52">
       <c r="A47" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -3610,7 +3611,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="21.75" customHeight="1" s="51">
+    <row r="48" ht="21.75" customHeight="1" s="52">
       <c r="A48" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -3637,7 +3638,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="30" customHeight="1" s="51">
+    <row r="49" ht="30" customHeight="1" s="52">
       <c r="A49" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -3664,30 +3665,30 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="21.75" customHeight="1" s="51">
-      <c r="A50" s="38" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B50" s="39" t="inlineStr">
+    <row r="50" ht="21.75" customHeight="1" s="52">
+      <c r="A50" s="36" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B50" s="37" t="inlineStr">
         <is>
           <t>QA-2.7-6</t>
         </is>
       </c>
-      <c r="C50" s="40" t="inlineStr">
+      <c r="C50" s="38" t="inlineStr">
         <is>
           <t>'Single user' send to unknown email → still sends and reports count: 1</t>
         </is>
       </c>
-      <c r="D50" s="41" t="n"/>
-      <c r="E50" s="42" t="inlineStr">
+      <c r="D50" s="39" t="n"/>
+      <c r="E50" s="40" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="21.75" customHeight="1" s="51">
+    <row r="51" ht="21.75" customHeight="1" s="52">
       <c r="A51" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -3708,14 +3709,14 @@
           <t>No issues</t>
         </is>
       </c>
-      <c r="E51" s="43" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="21.75" customHeight="1" s="51">
-      <c r="A52" s="44" t="inlineStr">
+      <c r="E51" s="41" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="21.75" customHeight="1" s="52">
+      <c r="A52" s="42" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
@@ -3735,13 +3736,13 @@
           <t>No issues</t>
         </is>
       </c>
-      <c r="E52" s="43" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="21.75" customHeight="1" s="51">
+      <c r="E52" s="41" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="21.75" customHeight="1" s="52">
       <c r="A53" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -3768,8 +3769,8 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="19.5" customHeight="1" s="51">
-      <c r="A55" s="54" t="inlineStr">
+    <row r="55" ht="19.5" customHeight="1" s="52">
+      <c r="A55" s="56" t="inlineStr">
         <is>
           <t xml:space="preserve">  2.8 Cross-cutting / Regression</t>
         </is>
@@ -3856,7 +3857,7 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="21.75" customHeight="1" s="51">
+    <row r="59" ht="21.75" customHeight="1" s="52">
       <c r="A59" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -3884,14 +3885,14 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="54" t="n"/>
+      <c r="A61" s="56" t="n"/>
       <c r="C61" t="inlineStr">
         <is>
           <t xml:space="preserve">  2.9 v2 - Categories, Test Cases &amp; the Audit Log</t>
         </is>
       </c>
     </row>
-    <row r="62" ht="22.8" customHeight="1" s="51">
+    <row r="62" ht="22.8" customHeight="1" s="52">
       <c r="A62" s="3" t="n"/>
       <c r="B62" s="8" t="inlineStr">
         <is>
@@ -3914,7 +3915,7 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="22.8" customHeight="1" s="51">
+    <row r="63" ht="22.8" customHeight="1" s="52">
       <c r="A63" s="3" t="n"/>
       <c r="B63" s="8" t="inlineStr">
         <is>
@@ -3937,7 +3938,7 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="22.8" customHeight="1" s="51">
+    <row r="64" ht="22.8" customHeight="1" s="52">
       <c r="A64" s="3" t="n"/>
       <c r="B64" s="8" t="inlineStr">
         <is>
@@ -3960,7 +3961,7 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="22.8" customHeight="1" s="51">
+    <row r="65" ht="22.8" customHeight="1" s="52">
       <c r="A65" s="3" t="n"/>
       <c r="B65" s="8" t="inlineStr">
         <is>
@@ -3983,7 +3984,7 @@
         </is>
       </c>
     </row>
-    <row r="66" ht="15" customHeight="1" s="51">
+    <row r="66" ht="15" customHeight="1" s="52">
       <c r="A66" s="3" t="n"/>
       <c r="B66" s="8" t="inlineStr">
         <is>
@@ -4006,7 +4007,7 @@
         </is>
       </c>
     </row>
-    <row r="67" ht="22.8" customHeight="1" s="51">
+    <row r="67" ht="22.8" customHeight="1" s="52">
       <c r="A67" s="3" t="n"/>
       <c r="B67" s="8" t="inlineStr">
         <is>
@@ -4029,7 +4030,7 @@
         </is>
       </c>
     </row>
-    <row r="68" ht="15" customHeight="1" s="51">
+    <row r="68" ht="15" customHeight="1" s="52">
       <c r="A68" s="3" t="n"/>
       <c r="B68" s="8" t="inlineStr">
         <is>
@@ -4052,7 +4053,7 @@
         </is>
       </c>
     </row>
-    <row r="69" ht="22.8" customHeight="1" s="51">
+    <row r="69" ht="22.8" customHeight="1" s="52">
       <c r="A69" s="3" t="n"/>
       <c r="B69" s="8" t="inlineStr">
         <is>
@@ -4075,7 +4076,7 @@
         </is>
       </c>
     </row>
-    <row r="70" ht="22.8" customHeight="1" s="51">
+    <row r="70" ht="22.8" customHeight="1" s="52">
       <c r="A70" s="3" t="n"/>
       <c r="B70" s="8" t="inlineStr">
         <is>
@@ -4098,7 +4099,7 @@
         </is>
       </c>
     </row>
-    <row r="71" ht="22.8" customHeight="1" s="51">
+    <row r="71" ht="22.8" customHeight="1" s="52">
       <c r="A71" s="3" t="n"/>
       <c r="B71" s="8" t="inlineStr">
         <is>
@@ -4121,7 +4122,7 @@
         </is>
       </c>
     </row>
-    <row r="72" ht="22.8" customHeight="1" s="51">
+    <row r="72" ht="22.8" customHeight="1" s="52">
       <c r="A72" s="3" t="n"/>
       <c r="B72" s="8" t="inlineStr">
         <is>
@@ -4144,7 +4145,7 @@
         </is>
       </c>
     </row>
-    <row r="73" ht="22.8" customHeight="1" s="51">
+    <row r="73" ht="22.8" customHeight="1" s="52">
       <c r="A73" s="3" t="n"/>
       <c r="B73" s="8" t="inlineStr">
         <is>
@@ -4167,7 +4168,7 @@
         </is>
       </c>
     </row>
-    <row r="74" ht="15" customHeight="1" s="51">
+    <row r="74" ht="15" customHeight="1" s="52">
       <c r="A74" s="3" t="n"/>
       <c r="B74" s="8" t="inlineStr">
         <is>
@@ -4186,7 +4187,7 @@
       </c>
       <c r="E74" s="7" t="n"/>
     </row>
-    <row r="75" ht="22.8" customHeight="1" s="51">
+    <row r="75" ht="22.8" customHeight="1" s="52">
       <c r="A75" s="3" t="n"/>
       <c r="B75" s="8" t="inlineStr">
         <is>
@@ -4209,7 +4210,7 @@
         </is>
       </c>
     </row>
-    <row r="76" ht="22.8" customHeight="1" s="51">
+    <row r="76" ht="22.8" customHeight="1" s="52">
       <c r="A76" s="3" t="n"/>
       <c r="B76" s="8" t="inlineStr">
         <is>
@@ -4229,14 +4230,14 @@
       <c r="E76" s="7" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="54" t="n"/>
+      <c r="A78" s="56" t="n"/>
       <c r="C78" t="inlineStr">
         <is>
           <t xml:space="preserve">  2.10 UX polish — error focus, focus rings, optional notes, audit fields</t>
         </is>
       </c>
     </row>
-    <row r="79" ht="34.2" customHeight="1" s="51">
+    <row r="79" ht="34.2" customHeight="1" s="52">
       <c r="A79" s="3" t="n"/>
       <c r="B79" s="8" t="inlineStr">
         <is>
@@ -4259,7 +4260,7 @@
         </is>
       </c>
     </row>
-    <row r="80" ht="22.8" customHeight="1" s="51">
+    <row r="80" ht="22.8" customHeight="1" s="52">
       <c r="A80" s="3" t="n"/>
       <c r="B80" s="8" t="inlineStr">
         <is>
@@ -4282,7 +4283,7 @@
         </is>
       </c>
     </row>
-    <row r="81" ht="15" customHeight="1" s="51">
+    <row r="81" ht="15" customHeight="1" s="52">
       <c r="A81" s="3" t="n"/>
       <c r="B81" s="8" t="inlineStr">
         <is>
@@ -4305,7 +4306,7 @@
         </is>
       </c>
     </row>
-    <row r="82" ht="22.8" customHeight="1" s="51">
+    <row r="82" ht="22.8" customHeight="1" s="52">
       <c r="A82" s="3" t="n"/>
       <c r="B82" s="8" t="inlineStr">
         <is>
@@ -4328,7 +4329,7 @@
         </is>
       </c>
     </row>
-    <row r="83" ht="22.8" customHeight="1" s="51">
+    <row r="83" ht="22.8" customHeight="1" s="52">
       <c r="A83" s="3" t="n"/>
       <c r="B83" s="8" t="inlineStr">
         <is>
@@ -4351,7 +4352,7 @@
         </is>
       </c>
     </row>
-    <row r="84" ht="22.8" customHeight="1" s="51">
+    <row r="84" ht="22.8" customHeight="1" s="52">
       <c r="A84" s="3" t="n"/>
       <c r="B84" s="8" t="inlineStr">
         <is>
@@ -4374,7 +4375,7 @@
         </is>
       </c>
     </row>
-    <row r="85" ht="34.2" customHeight="1" s="51">
+    <row r="85" ht="34.2" customHeight="1" s="52">
       <c r="A85" s="3" t="n"/>
       <c r="B85" s="8" t="inlineStr">
         <is>
@@ -4397,7 +4398,7 @@
         </is>
       </c>
     </row>
-    <row r="86" ht="22.8" customHeight="1" s="51">
+    <row r="86" ht="22.8" customHeight="1" s="52">
       <c r="A86" s="3" t="n"/>
       <c r="B86" s="8" t="inlineStr">
         <is>
@@ -4420,7 +4421,7 @@
         </is>
       </c>
     </row>
-    <row r="87" ht="15" customHeight="1" s="51">
+    <row r="87" ht="15" customHeight="1" s="52">
       <c r="A87" s="3" t="n"/>
       <c r="B87" s="8" t="inlineStr">
         <is>
@@ -4443,7 +4444,7 @@
         </is>
       </c>
     </row>
-    <row r="88" ht="22.8" customHeight="1" s="51">
+    <row r="88" ht="22.8" customHeight="1" s="52">
       <c r="A88" s="3" t="n"/>
       <c r="B88" s="8" t="inlineStr">
         <is>
@@ -4466,7 +4467,7 @@
         </is>
       </c>
     </row>
-    <row r="89" ht="22.8" customHeight="1" s="51">
+    <row r="89" ht="22.8" customHeight="1" s="52">
       <c r="A89" s="3" t="n"/>
       <c r="B89" s="8" t="inlineStr">
         <is>
@@ -4489,7 +4490,7 @@
         </is>
       </c>
     </row>
-    <row r="90" ht="22.8" customHeight="1" s="51">
+    <row r="90" ht="22.8" customHeight="1" s="52">
       <c r="A90" s="3" t="n"/>
       <c r="B90" s="8" t="inlineStr">
         <is>
@@ -4512,7 +4513,7 @@
         </is>
       </c>
     </row>
-    <row r="91" ht="22.8" customHeight="1" s="51">
+    <row r="91" ht="22.8" customHeight="1" s="52">
       <c r="A91" s="3" t="n"/>
       <c r="B91" s="8" t="inlineStr">
         <is>
@@ -4535,7 +4536,7 @@
         </is>
       </c>
     </row>
-    <row r="92" ht="22.8" customHeight="1" s="51">
+    <row r="92" ht="22.8" customHeight="1" s="52">
       <c r="A92" s="3" t="n"/>
       <c r="B92" s="8" t="inlineStr">
         <is>
@@ -4558,7 +4559,7 @@
         </is>
       </c>
     </row>
-    <row r="93" ht="22.8" customHeight="1" s="51">
+    <row r="93" ht="22.8" customHeight="1" s="52">
       <c r="A93" s="3" t="n"/>
       <c r="B93" s="8" t="inlineStr">
         <is>
@@ -4582,14 +4583,14 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="54" t="n"/>
+      <c r="A95" s="56" t="n"/>
       <c r="C95" t="inlineStr">
         <is>
           <t xml:space="preserve">  2.11 Bug fix round 1 — found on an Android phone</t>
         </is>
       </c>
     </row>
-    <row r="96" ht="34.2" customHeight="1" s="51">
+    <row r="96" ht="34.2" customHeight="1" s="52">
       <c r="A96" s="3" t="n"/>
       <c r="B96" s="8" t="inlineStr">
         <is>
@@ -4612,7 +4613,7 @@
         </is>
       </c>
     </row>
-    <row r="97" ht="22.8" customHeight="1" s="51">
+    <row r="97" ht="22.8" customHeight="1" s="52">
       <c r="A97" s="3" t="n"/>
       <c r="B97" s="8" t="inlineStr">
         <is>
@@ -4635,7 +4636,7 @@
         </is>
       </c>
     </row>
-    <row r="98" ht="22.8" customHeight="1" s="51">
+    <row r="98" ht="22.8" customHeight="1" s="52">
       <c r="A98" s="3" t="n"/>
       <c r="B98" s="8" t="inlineStr">
         <is>
@@ -4658,7 +4659,7 @@
         </is>
       </c>
     </row>
-    <row r="99" ht="34.2" customHeight="1" s="51">
+    <row r="99" ht="34.2" customHeight="1" s="52">
       <c r="A99" s="3" t="n"/>
       <c r="B99" s="8" t="inlineStr">
         <is>
@@ -4681,7 +4682,7 @@
         </is>
       </c>
     </row>
-    <row r="100" ht="34.2" customHeight="1" s="51">
+    <row r="100" ht="34.2" customHeight="1" s="52">
       <c r="A100" s="3" t="n"/>
       <c r="B100" s="8" t="inlineStr">
         <is>
@@ -4704,7 +4705,7 @@
         </is>
       </c>
     </row>
-    <row r="101" ht="22.8" customHeight="1" s="51">
+    <row r="101" ht="22.8" customHeight="1" s="52">
       <c r="A101" s="3" t="n"/>
       <c r="B101" s="8" t="inlineStr">
         <is>
@@ -4727,7 +4728,7 @@
         </is>
       </c>
     </row>
-    <row r="102" ht="22.8" customHeight="1" s="51">
+    <row r="102" ht="22.8" customHeight="1" s="52">
       <c r="A102" s="3" t="n"/>
       <c r="B102" s="8" t="inlineStr">
         <is>
@@ -4750,7 +4751,7 @@
         </is>
       </c>
     </row>
-    <row r="103" ht="22.8" customHeight="1" s="51">
+    <row r="103" ht="22.8" customHeight="1" s="52">
       <c r="A103" s="3" t="n"/>
       <c r="B103" s="8" t="inlineStr">
         <is>
@@ -4773,7 +4774,7 @@
         </is>
       </c>
     </row>
-    <row r="104" ht="22.8" customHeight="1" s="51">
+    <row r="104" ht="22.8" customHeight="1" s="52">
       <c r="A104" s="3" t="n"/>
       <c r="B104" s="8" t="inlineStr">
         <is>
@@ -4796,7 +4797,7 @@
         </is>
       </c>
     </row>
-    <row r="105" ht="34.2" customHeight="1" s="51">
+    <row r="105" ht="34.2" customHeight="1" s="52">
       <c r="A105" s="3" t="n"/>
       <c r="B105" s="8" t="inlineStr">
         <is>
@@ -4819,7 +4820,7 @@
         </is>
       </c>
     </row>
-    <row r="106" ht="34.2" customHeight="1" s="51">
+    <row r="106" ht="34.2" customHeight="1" s="52">
       <c r="A106" s="3" t="n"/>
       <c r="B106" s="8" t="inlineStr">
         <is>
@@ -4842,7 +4843,7 @@
         </is>
       </c>
     </row>
-    <row r="107" ht="34.2" customHeight="1" s="51">
+    <row r="107" ht="34.2" customHeight="1" s="52">
       <c r="A107" s="3" t="n"/>
       <c r="B107" s="8" t="inlineStr">
         <is>
@@ -4865,7 +4866,7 @@
         </is>
       </c>
     </row>
-    <row r="108" ht="22.8" customHeight="1" s="51">
+    <row r="108" ht="22.8" customHeight="1" s="52">
       <c r="A108" s="3" t="n"/>
       <c r="B108" s="8" t="inlineStr">
         <is>
@@ -4889,14 +4890,14 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="54" t="n"/>
+      <c r="A110" s="56" t="n"/>
       <c r="C110" t="inlineStr">
         <is>
           <t xml:space="preserve">  2.12 AI shadow metering — ai_usage_events</t>
         </is>
       </c>
     </row>
-    <row r="111" ht="34.2" customHeight="1" s="51">
+    <row r="111" ht="34.2" customHeight="1" s="52">
       <c r="A111" s="3" t="n"/>
       <c r="B111" s="8" t="inlineStr">
         <is>
@@ -4915,7 +4916,7 @@
       </c>
       <c r="E111" s="7" t="n"/>
     </row>
-    <row r="112" ht="34.2" customHeight="1" s="51">
+    <row r="112" ht="34.2" customHeight="1" s="52">
       <c r="A112" s="3" t="n"/>
       <c r="B112" s="8" t="inlineStr">
         <is>
@@ -4935,14 +4936,14 @@
       <c r="E112" s="7" t="n"/>
     </row>
     <row r="113">
-      <c r="A113" s="54" t="n"/>
+      <c r="A113" s="56" t="n"/>
       <c r="C113" t="inlineStr">
         <is>
           <t xml:space="preserve">  2.13 Report allowance — publish, cap, release</t>
         </is>
       </c>
     </row>
-    <row r="114" ht="34.2" customHeight="1" s="51">
+    <row r="114" ht="34.2" customHeight="1" s="52">
       <c r="A114" s="3" t="n"/>
       <c r="B114" s="8" t="inlineStr">
         <is>
@@ -4965,7 +4966,7 @@
         </is>
       </c>
     </row>
-    <row r="115" ht="34.2" customHeight="1" s="51">
+    <row r="115" ht="34.2" customHeight="1" s="52">
       <c r="A115" s="3" t="n"/>
       <c r="B115" s="8" t="inlineStr">
         <is>
@@ -4988,7 +4989,7 @@
         </is>
       </c>
     </row>
-    <row r="116" ht="34.2" customHeight="1" s="51">
+    <row r="116" ht="34.2" customHeight="1" s="52">
       <c r="A116" s="3" t="n"/>
       <c r="B116" s="8" t="inlineStr">
         <is>
@@ -5011,7 +5012,7 @@
         </is>
       </c>
     </row>
-    <row r="117" ht="22.8" customHeight="1" s="51">
+    <row r="117" ht="22.8" customHeight="1" s="52">
       <c r="A117" s="3" t="n"/>
       <c r="B117" s="8" t="inlineStr">
         <is>
@@ -5030,7 +5031,7 @@
       </c>
       <c r="E117" s="7" t="n"/>
     </row>
-    <row r="118" ht="34.2" customHeight="1" s="51">
+    <row r="118" ht="34.2" customHeight="1" s="52">
       <c r="A118" s="3" t="n"/>
       <c r="B118" s="8" t="inlineStr">
         <is>
@@ -5053,7 +5054,7 @@
         </is>
       </c>
     </row>
-    <row r="119" ht="15" customHeight="1" s="51">
+    <row r="119" ht="15" customHeight="1" s="52">
       <c r="A119" s="3" t="n"/>
       <c r="B119" s="8" t="inlineStr">
         <is>
@@ -5076,7 +5077,7 @@
         </is>
       </c>
     </row>
-    <row r="120" ht="22.8" customHeight="1" s="51">
+    <row r="120" ht="22.8" customHeight="1" s="52">
       <c r="A120" s="3" t="n"/>
       <c r="B120" s="8" t="inlineStr">
         <is>
@@ -5099,7 +5100,7 @@
         </is>
       </c>
     </row>
-    <row r="121" ht="22.8" customHeight="1" s="51">
+    <row r="121" ht="22.8" customHeight="1" s="52">
       <c r="A121" s="3" t="n"/>
       <c r="B121" s="8" t="inlineStr">
         <is>
@@ -5122,7 +5123,7 @@
         </is>
       </c>
     </row>
-    <row r="122" ht="15" customHeight="1" s="51">
+    <row r="122" ht="15" customHeight="1" s="52">
       <c r="A122" s="3" t="n"/>
       <c r="B122" s="8" t="inlineStr">
         <is>
@@ -5142,14 +5143,14 @@
       <c r="E122" s="7" t="n"/>
     </row>
     <row r="123">
-      <c r="A123" s="54" t="n"/>
+      <c r="A123" s="56" t="n"/>
       <c r="C123" t="inlineStr">
         <is>
           <t xml:space="preserve">  2.14 One report per mission</t>
         </is>
       </c>
     </row>
-    <row r="124" ht="34.2" customHeight="1" s="51">
+    <row r="124" ht="34.2" customHeight="1" s="52">
       <c r="A124" s="3" t="n"/>
       <c r="B124" s="8" t="inlineStr">
         <is>
@@ -5172,7 +5173,7 @@
         </is>
       </c>
     </row>
-    <row r="125" ht="15" customHeight="1" s="51">
+    <row r="125" ht="15" customHeight="1" s="52">
       <c r="A125" s="3" t="n"/>
       <c r="B125" s="8" t="inlineStr">
         <is>
@@ -5196,14 +5197,14 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="54" t="n"/>
+      <c r="A126" s="56" t="n"/>
       <c r="C126" t="inlineStr">
         <is>
           <t xml:space="preserve">  2.15 Cohort payouts</t>
         </is>
       </c>
     </row>
-    <row r="127" ht="34.2" customHeight="1" s="51">
+    <row r="127" ht="34.2" customHeight="1" s="52">
       <c r="A127" s="3" t="n"/>
       <c r="B127" s="8" t="inlineStr">
         <is>
@@ -5222,7 +5223,7 @@
       </c>
       <c r="E127" s="7" t="n"/>
     </row>
-    <row r="128" ht="22.8" customHeight="1" s="51">
+    <row r="128" ht="22.8" customHeight="1" s="52">
       <c r="A128" s="3" t="n"/>
       <c r="B128" s="8" t="inlineStr">
         <is>
@@ -5241,7 +5242,7 @@
       </c>
       <c r="E128" s="7" t="n"/>
     </row>
-    <row r="129" ht="34.2" customHeight="1" s="51">
+    <row r="129" ht="34.2" customHeight="1" s="52">
       <c r="A129" s="3" t="n"/>
       <c r="B129" s="8" t="inlineStr">
         <is>
@@ -5260,7 +5261,7 @@
       </c>
       <c r="E129" s="7" t="n"/>
     </row>
-    <row r="130" ht="22.8" customHeight="1" s="51">
+    <row r="130" ht="22.8" customHeight="1" s="52">
       <c r="A130" s="3" t="n"/>
       <c r="B130" s="8" t="inlineStr">
         <is>
@@ -5279,7 +5280,7 @@
       </c>
       <c r="E130" s="7" t="n"/>
     </row>
-    <row r="131" ht="22.8" customHeight="1" s="51">
+    <row r="131" ht="22.8" customHeight="1" s="52">
       <c r="A131" s="3" t="n"/>
       <c r="B131" s="8" t="inlineStr">
         <is>
@@ -5298,7 +5299,7 @@
       </c>
       <c r="E131" s="7" t="n"/>
     </row>
-    <row r="132" ht="15" customHeight="1" s="51">
+    <row r="132" ht="15" customHeight="1" s="52">
       <c r="A132" s="3" t="n"/>
       <c r="B132" s="8" t="inlineStr">
         <is>
@@ -5317,15 +5318,15 @@
       </c>
       <c r="E132" s="7" t="n"/>
     </row>
-    <row r="133" s="51">
-      <c r="A133" s="54" t="n"/>
+    <row r="133">
+      <c r="A133" s="56" t="n"/>
       <c r="C133" t="inlineStr">
         <is>
           <t xml:space="preserve">  2.16 Rate limiting</t>
         </is>
       </c>
     </row>
-    <row r="134" ht="45.6" customHeight="1" s="51">
+    <row r="134" ht="45.6" customHeight="1" s="52">
       <c r="A134" s="3" t="n"/>
       <c r="B134" s="8" t="inlineStr">
         <is>
@@ -5344,7 +5345,7 @@
       </c>
       <c r="E134" s="7" t="n"/>
     </row>
-    <row r="135" ht="22.8" customHeight="1" s="51">
+    <row r="135" ht="22.8" customHeight="1" s="52">
       <c r="A135" s="3" t="n"/>
       <c r="B135" s="8" t="inlineStr">
         <is>
@@ -5363,7 +5364,7 @@
       </c>
       <c r="E135" s="7" t="n"/>
     </row>
-    <row r="136" ht="34.2" customHeight="1" s="51">
+    <row r="136" ht="34.2" customHeight="1" s="52">
       <c r="A136" s="3" t="n"/>
       <c r="B136" s="8" t="inlineStr">
         <is>
@@ -5382,7 +5383,7 @@
       </c>
       <c r="E136" s="7" t="n"/>
     </row>
-    <row r="137" ht="34.2" customHeight="1" s="51">
+    <row r="137" ht="34.2" customHeight="1" s="52">
       <c r="A137" s="3" t="n"/>
       <c r="B137" s="8" t="inlineStr">
         <is>
@@ -5401,7 +5402,7 @@
       </c>
       <c r="E137" s="7" t="n"/>
     </row>
-    <row r="138" ht="34.2" customHeight="1" s="51">
+    <row r="138" ht="34.2" customHeight="1" s="52">
       <c r="A138" s="3" t="n"/>
       <c r="B138" s="8" t="inlineStr">
         <is>
@@ -5421,14 +5422,14 @@
       <c r="E138" s="7" t="n"/>
     </row>
     <row r="139">
-      <c r="A139" s="54" t="n"/>
+      <c r="A139" s="56" t="n"/>
       <c r="C139" t="inlineStr">
         <is>
           <t xml:space="preserve">  2.17 Tester anonymity</t>
         </is>
       </c>
     </row>
-    <row r="140" ht="45.6" customHeight="1" s="51">
+    <row r="140" ht="45.6" customHeight="1" s="52">
       <c r="A140" s="3" t="n"/>
       <c r="B140" s="8" t="inlineStr">
         <is>
@@ -5445,9 +5446,13 @@
           <t>New in tester anonymity</t>
         </is>
       </c>
-      <c r="E140" s="7" t="n"/>
-    </row>
-    <row r="141" ht="45.6" customHeight="1" s="51">
+      <c r="E140" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="45.6" customHeight="1" s="52">
       <c r="A141" s="3" t="n"/>
       <c r="B141" s="8" t="inlineStr">
         <is>
@@ -5456,7 +5461,7 @@
       </c>
       <c r="C141" s="9" t="inlineStr">
         <is>
-          <t>Export the feedback CSV across two missions: the column reads "Tester # (per mission)", holds numbers not names, restarts at 1 on each mission, and matches the "Tester N" on the mission page. A second export gives the same numbers.</t>
+          <t>Settings → Account → Export: pick a project and leave Mission on "All missions — one sheet each" → an .xlsx named for the project downloads, with one sheet per mission (named for it). Tester # restarts at 1 on each sheet and matches "Tester N" on the mission page; no names anywhere.</t>
         </is>
       </c>
       <c r="D141" s="23" t="inlineStr">
@@ -5466,7 +5471,7 @@
       </c>
       <c r="E141" s="7" t="n"/>
     </row>
-    <row r="142" ht="45.6" customHeight="1" s="51">
+    <row r="142" ht="45.6" customHeight="1" s="52">
       <c r="A142" s="3" t="n"/>
       <c r="B142" s="8" t="inlineStr">
         <is>
@@ -5485,7 +5490,7 @@
       </c>
       <c r="E142" s="7" t="n"/>
     </row>
-    <row r="143" ht="45.6" customHeight="1" s="51">
+    <row r="143" ht="45.6" customHeight="1" s="52">
       <c r="A143" s="3" t="n"/>
       <c r="B143" s="8" t="inlineStr">
         <is>
@@ -5502,9 +5507,13 @@
           <t>New in tester anonymity</t>
         </is>
       </c>
-      <c r="E143" s="7" t="n"/>
-    </row>
-    <row r="144" ht="45.6" customHeight="1" s="51">
+      <c r="E143" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="45.6" customHeight="1" s="52">
       <c r="A144" s="3" t="n"/>
       <c r="B144" s="8" t="inlineStr">
         <is>
@@ -5521,9 +5530,13 @@
           <t>New in tester anonymity</t>
         </is>
       </c>
-      <c r="E144" s="7" t="n"/>
-    </row>
-    <row r="145" ht="45.6" customHeight="1" s="51">
+      <c r="E144" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="45.6" customHeight="1" s="52">
       <c r="A145" s="3" t="n"/>
       <c r="B145" s="8" t="inlineStr">
         <is>
@@ -5540,9 +5553,13 @@
           <t>New in tester anonymity</t>
         </is>
       </c>
-      <c r="E145" s="7" t="n"/>
-    </row>
-    <row r="146" ht="45.6" customHeight="1" s="51">
+      <c r="E145" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="45.6" customHeight="1" s="52">
       <c r="A146" s="3" t="n"/>
       <c r="B146" s="8" t="inlineStr">
         <is>
@@ -5559,7 +5576,30 @@
           <t>New in tester anonymity</t>
         </is>
       </c>
-      <c r="E146" s="7" t="n"/>
+      <c r="E146" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="3" t="n"/>
+      <c r="B147" s="8" t="inlineStr">
+        <is>
+          <t>QA-2.17-8</t>
+        </is>
+      </c>
+      <c r="C147" s="9" t="inlineStr">
+        <is>
+          <t>Pick one mission in the Mission select → the button reads "Download CSV" and a CSV for just that mission downloads, named project-mission-date.csv. Switching project resets Mission to "All missions". A project with no reports is not offered.</t>
+        </is>
+      </c>
+      <c r="D147" s="23" t="inlineStr">
+        <is>
+          <t>New in tester anonymity</t>
+        </is>
+      </c>
+      <c r="E147" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -5682,22 +5722,22 @@
   <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
-    <col width="5" customWidth="1" style="51" min="1" max="1"/>
-    <col width="12" customWidth="1" style="51" min="2" max="2"/>
-    <col width="58" customWidth="1" style="51" min="3" max="3"/>
-    <col width="36" customWidth="1" style="51" min="4" max="4"/>
-    <col width="14" customWidth="1" style="51" min="5" max="5"/>
+    <col width="5" customWidth="1" style="52" min="1" max="1"/>
+    <col width="12" customWidth="1" style="52" min="2" max="2"/>
+    <col width="58" customWidth="1" style="52" min="3" max="3"/>
+    <col width="36" customWidth="1" style="52" min="4" max="4"/>
+    <col width="14" customWidth="1" style="52" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" s="51">
-      <c r="A1" s="57" t="inlineStr">
+    <row r="1" ht="31.5" customHeight="1" s="52">
+      <c r="A1" s="58" t="inlineStr">
         <is>
           <t>TownHall — 3 · End-User Sanity</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="19.5" customHeight="1" s="51">
-      <c r="A2" s="53">
+    <row r="2" ht="19.5" customHeight="1" s="52">
+      <c r="A2" s="54">
         <f>IFERROR(COUNTIF(E4:E2000,"Done")&amp;" / "&amp;COUNTA(B4:B2000)&amp;" items completed","0 / 0 items completed")</f>
         <v/>
       </c>
@@ -5706,7 +5746,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="21.75" customHeight="1" s="51">
+    <row r="3" ht="21.75" customHeight="1" s="52">
       <c r="A3" s="14" t="n"/>
       <c r="B3" s="14" t="inlineStr">
         <is>
@@ -5729,14 +5769,14 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="19.5" customHeight="1" s="51">
-      <c r="A4" s="56" t="inlineStr">
+    <row r="4" ht="19.5" customHeight="1" s="52">
+      <c r="A4" s="57" t="inlineStr">
         <is>
           <t xml:space="preserve">  3.1 As a Developer-User</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1" s="51">
+    <row r="5" ht="30" customHeight="1" s="52">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -5763,7 +5803,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1" s="51">
+    <row r="6" ht="30" customHeight="1" s="52">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -5790,7 +5830,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="30" customHeight="1" s="51">
+    <row r="7" ht="30" customHeight="1" s="52">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -5817,7 +5857,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="30" customHeight="1" s="51">
+    <row r="8" ht="30" customHeight="1" s="52">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -5844,7 +5884,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1" s="51">
+    <row r="9" ht="30" customHeight="1" s="52">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -5871,7 +5911,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="30" customHeight="1" s="51">
+    <row r="10" ht="30" customHeight="1" s="52">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -5898,7 +5938,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1" s="51">
+    <row r="11" ht="30" customHeight="1" s="52">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -5925,7 +5965,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="30" customHeight="1" s="51">
+    <row r="12" ht="30" customHeight="1" s="52">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -5952,14 +5992,14 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="19.5" customHeight="1" s="51">
-      <c r="A14" s="56" t="inlineStr">
+    <row r="14" ht="19.5" customHeight="1" s="52">
+      <c r="A14" s="57" t="inlineStr">
         <is>
           <t xml:space="preserve">  3.2 As a Tester-User</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="21.75" customHeight="1" s="51">
+    <row r="15" ht="21.75" customHeight="1" s="52">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -5986,7 +6026,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="30" customHeight="1" s="51">
+    <row r="16" ht="30" customHeight="1" s="52">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -6013,7 +6053,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="30" customHeight="1" s="51">
+    <row r="17" ht="30" customHeight="1" s="52">
       <c r="A17" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -6036,7 +6076,7 @@
       </c>
       <c r="E17" s="7" t="n"/>
     </row>
-    <row r="18" ht="30" customHeight="1" s="51">
+    <row r="18" ht="30" customHeight="1" s="52">
       <c r="A18" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -6063,7 +6103,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="30" customHeight="1" s="51">
+    <row r="19" ht="30" customHeight="1" s="52">
       <c r="A19" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -6090,14 +6130,14 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="19.5" customHeight="1" s="51">
-      <c r="A21" s="56" t="inlineStr">
+    <row r="21" ht="19.5" customHeight="1" s="52">
+      <c r="A21" s="57" t="inlineStr">
         <is>
           <t xml:space="preserve">  3.3 As an Admin</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="21.75" customHeight="1" s="51">
+    <row r="22" ht="21.75" customHeight="1" s="52">
       <c r="A22" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -6120,7 +6160,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="30" customHeight="1" s="51">
+    <row r="23" ht="30" customHeight="1" s="52">
       <c r="A23" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -6147,7 +6187,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="30" customHeight="1" s="51">
+    <row r="24" ht="30" customHeight="1" s="52">
       <c r="A24" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -6170,7 +6210,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="30" customHeight="1" s="51">
+    <row r="25" ht="30" customHeight="1" s="52">
       <c r="A25" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -6194,13 +6234,13 @@
       </c>
     </row>
     <row r="27">
-      <c r="C27" s="56" t="inlineStr">
+      <c r="C27" s="57" t="inlineStr">
         <is>
           <t xml:space="preserve">  3.4 v2 - As a Tester and Builder</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="22.8" customHeight="1" s="51">
+    <row r="28" ht="22.8" customHeight="1" s="52">
       <c r="A28" s="3" t="n"/>
       <c r="B28" s="4" t="inlineStr">
         <is>
@@ -6223,7 +6263,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="15" customHeight="1" s="51">
+    <row r="29" ht="15" customHeight="1" s="52">
       <c r="A29" s="3" t="n"/>
       <c r="B29" s="4" t="inlineStr">
         <is>
@@ -6307,22 +6347,22 @@
   <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
-    <col width="5" customWidth="1" style="51" min="1" max="1"/>
-    <col width="12" customWidth="1" style="51" min="2" max="2"/>
-    <col width="58" customWidth="1" style="51" min="3" max="3"/>
-    <col width="36" customWidth="1" style="51" min="4" max="4"/>
-    <col width="14" customWidth="1" style="51" min="5" max="5"/>
+    <col width="5" customWidth="1" style="52" min="1" max="1"/>
+    <col width="12" customWidth="1" style="52" min="2" max="2"/>
+    <col width="58" customWidth="1" style="52" min="3" max="3"/>
+    <col width="36" customWidth="1" style="52" min="4" max="4"/>
+    <col width="14" customWidth="1" style="52" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" s="51">
-      <c r="A1" s="58" t="inlineStr">
+    <row r="1" ht="31.5" customHeight="1" s="52">
+      <c r="A1" s="59" t="inlineStr">
         <is>
           <t>TownHall — 4 · Release Checklist</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="19.5" customHeight="1" s="51">
-      <c r="A2" s="53">
+    <row r="2" ht="19.5" customHeight="1" s="52">
+      <c r="A2" s="54">
         <f>IFERROR(COUNTIF(E4:E2000,"Done")&amp;" / "&amp;COUNTA(B4:B2000)&amp;" items completed","0 / 0 items completed")</f>
         <v/>
       </c>
@@ -6331,7 +6371,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="21.75" customHeight="1" s="51">
+    <row r="3" ht="21.75" customHeight="1" s="52">
       <c r="A3" s="16" t="n"/>
       <c r="B3" s="16" t="inlineStr">
         <is>
@@ -6354,14 +6394,14 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="19.5" customHeight="1" s="51">
-      <c r="A4" s="59" t="inlineStr">
+    <row r="4" ht="19.5" customHeight="1" s="52">
+      <c r="A4" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">  5. Release Checklist — Before merging to main</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="21.75" customHeight="1" s="51">
+    <row r="5" ht="21.75" customHeight="1" s="52">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -6388,7 +6428,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="21.75" customHeight="1" s="51">
+    <row r="6" ht="21.75" customHeight="1" s="52">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -6415,7 +6455,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="30" customHeight="1" s="51">
+    <row r="7" ht="30" customHeight="1" s="52">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -6442,7 +6482,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="21.75" customHeight="1" s="51">
+    <row r="8" ht="21.75" customHeight="1" s="52">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -6469,7 +6509,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="21.75" customHeight="1" s="51">
+    <row r="9" ht="21.75" customHeight="1" s="52">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -6496,7 +6536,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="21.75" customHeight="1" s="51">
+    <row r="10" ht="21.75" customHeight="1" s="52">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -6523,14 +6563,14 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="19.5" customHeight="1" s="51">
-      <c r="A12" s="59" t="inlineStr">
+    <row r="12" ht="19.5" customHeight="1" s="52">
+      <c r="A12" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">  Environment — Verify before E2E run</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="21.75" customHeight="1" s="51">
+    <row r="13" ht="21.75" customHeight="1" s="52">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -6557,7 +6597,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="21.75" customHeight="1" s="51">
+    <row r="14" ht="21.75" customHeight="1" s="52">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -6580,7 +6620,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="21.75" customHeight="1" s="51">
+    <row r="15" ht="21.75" customHeight="1" s="52">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -6603,7 +6643,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="21.75" customHeight="1" s="51">
+    <row r="16" ht="21.75" customHeight="1" s="52">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -6626,7 +6666,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="21.75" customHeight="1" s="51">
+    <row r="17" ht="21.75" customHeight="1" s="52">
       <c r="A17" s="3" t="inlineStr">
         <is>
           <t>☐</t>
@@ -6653,7 +6693,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1" s="51">
+    <row r="18" ht="30" customHeight="1" s="52">
       <c r="A18" s="3" t="inlineStr">
         <is>
           <t>☐</t>

</xml_diff>

<commit_message>
Add the 2.18 approval notification checklist rows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TownHall_Checklist (1).xlsx
+++ b/TownHall_Checklist (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\townhall\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C64C56C-6CFF-4F92-8EAB-B21DF7A3A652}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{728E0783-B22C-4E0C-B148-3F06628C4F3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="908" uniqueCount="505">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="926" uniqueCount="515">
   <si>
     <t>TownHall — 1 · Engineer Tests</t>
   </si>
@@ -1312,6 +1312,36 @@
   </si>
   <si>
     <t>Pick one mission in the Mission select → the button reads "Download CSV" and a CSV for just that mission downloads, named project-mission-date.csv. Switching project resets Mission to "All missions". A project with no reports is not offered.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  2.18 Approval notification</t>
+  </si>
+  <si>
+    <t>QA-2.18-1</t>
+  </si>
+  <si>
+    <t>Approve a report with a rating and a note → the tester gets "Your report on “&lt;mission&gt;” was approved" in a real inbox, rendering the mission, "N out of 5", the note and a working View your reports link.</t>
+  </si>
+  <si>
+    <t>New in approval notification</t>
+  </si>
+  <si>
+    <t>QA-2.18-2</t>
+  </si>
+  <si>
+    <t>Approve with a rating of 1 and no note → the copy reads neutral, not sarcastic, and there is no "Note from the builder" block.</t>
+  </si>
+  <si>
+    <t>QA-2.18-3</t>
+  </si>
+  <si>
+    <t>With a bad RESEND_API_KEY, approve a report → the builder sees no error, the row shows Approved with its rating on the mission page and on the tester's /tester feed.</t>
+  </si>
+  <si>
+    <t>QA-2.18-4</t>
+  </si>
+  <si>
+    <t>The approval note shows under the approved row on the builder's mission page and on the tester's /tester feed row.</t>
   </si>
   <si>
     <t>TownHall — 3 · End-User Sanity</t>
@@ -3663,8 +3693,8 @@
   <mergeCells count="11">
     <mergeCell ref="A63:E63"/>
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:D2"/>
     <mergeCell ref="A13:E13"/>
-    <mergeCell ref="A2:D2"/>
     <mergeCell ref="A58:E58"/>
     <mergeCell ref="A53:E53"/>
     <mergeCell ref="A34:E34"/>
@@ -3785,7 +3815,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E147"/>
+  <dimension ref="A1:E152"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" style="48" customWidth="1"/>
@@ -3807,14 +3837,14 @@
     <row r="2" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="54" t="str">
         <f>IFERROR(COUNTIF(E4:E2000,"Done")&amp;" / "&amp;COUNTA(B4:B2000)&amp;" items completed","0 / 0 items completed")</f>
-        <v>92 / 116 items completed</v>
+        <v>97 / 120 items completed</v>
       </c>
       <c r="B2" s="52"/>
       <c r="C2" s="52"/>
       <c r="D2" s="52"/>
       <c r="E2" s="11">
         <f>IFERROR(COUNTIF(E4:E2000,"Done")/COUNTA(B4:B2000),0)</f>
-        <v>0.7931034482758621</v>
+        <v>0.80833333333333335</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -5642,7 +5672,9 @@
       <c r="D141" s="23" t="s">
         <v>410</v>
       </c>
-      <c r="E141" s="7"/>
+      <c r="E141" s="7" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="142" spans="1:5" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A142" s="3"/>
@@ -5655,7 +5687,9 @@
       <c r="D142" s="23" t="s">
         <v>410</v>
       </c>
-      <c r="E142" s="7"/>
+      <c r="E142" s="7" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="143" spans="1:5" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A143" s="3"/>
@@ -5717,7 +5751,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="147" spans="1:5" ht="45.6" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:5" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A147" s="3"/>
       <c r="B147" s="8" t="s">
         <v>423</v>
@@ -5729,6 +5763,70 @@
         <v>410</v>
       </c>
       <c r="E147" s="7" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A148" s="49"/>
+      <c r="C148" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="149" spans="1:5" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A149" s="3"/>
+      <c r="B149" s="8" t="s">
+        <v>426</v>
+      </c>
+      <c r="C149" s="9" t="s">
+        <v>427</v>
+      </c>
+      <c r="D149" s="23" t="s">
+        <v>428</v>
+      </c>
+      <c r="E149" s="7" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A150" s="3"/>
+      <c r="B150" s="8" t="s">
+        <v>429</v>
+      </c>
+      <c r="C150" s="9" t="s">
+        <v>430</v>
+      </c>
+      <c r="D150" s="23" t="s">
+        <v>428</v>
+      </c>
+      <c r="E150" s="7" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A151" s="3"/>
+      <c r="B151" s="8" t="s">
+        <v>431</v>
+      </c>
+      <c r="C151" s="9" t="s">
+        <v>432</v>
+      </c>
+      <c r="D151" s="23" t="s">
+        <v>428</v>
+      </c>
+      <c r="E151" s="7"/>
+    </row>
+    <row r="152" spans="1:5" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A152" s="3"/>
+      <c r="B152" s="8" t="s">
+        <v>433</v>
+      </c>
+      <c r="C152" s="9" t="s">
+        <v>434</v>
+      </c>
+      <c r="D152" s="23" t="s">
+        <v>428</v>
+      </c>
+      <c r="E152" s="7" t="s">
         <v>159</v>
       </c>
     </row>
@@ -5858,7 +5956,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="58" t="s">
-        <v>425</v>
+        <v>435</v>
       </c>
       <c r="B1" s="52"/>
       <c r="C1" s="52"/>
@@ -5895,7 +5993,7 @@
     </row>
     <row r="4" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="57" t="s">
-        <v>426</v>
+        <v>436</v>
       </c>
       <c r="B4" s="52"/>
       <c r="C4" s="52"/>
@@ -5907,10 +6005,10 @@
         <v>6</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>427</v>
+        <v>437</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>428</v>
+        <v>438</v>
       </c>
       <c r="D5" s="24" t="s">
         <v>158</v>
@@ -5924,10 +6022,10 @@
         <v>6</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>429</v>
+        <v>439</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>430</v>
+        <v>440</v>
       </c>
       <c r="D6" s="24" t="s">
         <v>158</v>
@@ -5941,10 +6039,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>431</v>
+        <v>441</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>432</v>
+        <v>442</v>
       </c>
       <c r="D7" s="24" t="s">
         <v>158</v>
@@ -5958,10 +6056,10 @@
         <v>6</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>433</v>
+        <v>443</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>434</v>
+        <v>444</v>
       </c>
       <c r="D8" s="24" t="s">
         <v>158</v>
@@ -5975,10 +6073,10 @@
         <v>6</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>435</v>
+        <v>445</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>436</v>
+        <v>446</v>
       </c>
       <c r="D9" s="24" t="s">
         <v>158</v>
@@ -5992,10 +6090,10 @@
         <v>6</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>437</v>
+        <v>447</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>438</v>
+        <v>448</v>
       </c>
       <c r="D10" s="24" t="s">
         <v>158</v>
@@ -6009,10 +6107,10 @@
         <v>6</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>439</v>
+        <v>449</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>440</v>
+        <v>450</v>
       </c>
       <c r="D11" s="24" t="s">
         <v>158</v>
@@ -6026,10 +6124,10 @@
         <v>6</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>441</v>
+        <v>451</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>442</v>
+        <v>452</v>
       </c>
       <c r="D12" s="24" t="s">
         <v>158</v>
@@ -6040,7 +6138,7 @@
     </row>
     <row r="14" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="57" t="s">
-        <v>443</v>
+        <v>453</v>
       </c>
       <c r="B14" s="52"/>
       <c r="C14" s="52"/>
@@ -6052,10 +6150,10 @@
         <v>6</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>444</v>
+        <v>454</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>445</v>
+        <v>455</v>
       </c>
       <c r="D15" s="34" t="s">
         <v>158</v>
@@ -6069,10 +6167,10 @@
         <v>6</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>446</v>
+        <v>456</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>447</v>
+        <v>457</v>
       </c>
       <c r="D16" s="34" t="s">
         <v>158</v>
@@ -6086,13 +6184,13 @@
         <v>6</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>449</v>
+        <v>459</v>
       </c>
       <c r="D17" s="34" t="s">
-        <v>450</v>
+        <v>460</v>
       </c>
       <c r="E17" s="7"/>
     </row>
@@ -6101,10 +6199,10 @@
         <v>6</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>451</v>
+        <v>461</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>452</v>
+        <v>462</v>
       </c>
       <c r="D18" s="34" t="s">
         <v>158</v>
@@ -6118,10 +6216,10 @@
         <v>6</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>453</v>
+        <v>463</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>454</v>
+        <v>464</v>
       </c>
       <c r="D19" s="34" t="s">
         <v>158</v>
@@ -6132,7 +6230,7 @@
     </row>
     <row r="21" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="57" t="s">
-        <v>455</v>
+        <v>465</v>
       </c>
       <c r="B21" s="52"/>
       <c r="C21" s="52"/>
@@ -6144,10 +6242,10 @@
         <v>6</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>456</v>
+        <v>466</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>457</v>
+        <v>467</v>
       </c>
       <c r="D22" s="10"/>
       <c r="E22" s="7" t="s">
@@ -6159,13 +6257,13 @@
         <v>6</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>458</v>
+        <v>468</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>459</v>
+        <v>469</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>460</v>
+        <v>470</v>
       </c>
       <c r="E23" s="7" t="s">
         <v>10</v>
@@ -6176,10 +6274,10 @@
         <v>6</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>461</v>
+        <v>471</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>462</v>
+        <v>472</v>
       </c>
       <c r="D24" s="10"/>
       <c r="E24" s="7" t="s">
@@ -6191,10 +6289,10 @@
         <v>6</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>463</v>
+        <v>473</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>464</v>
+        <v>474</v>
       </c>
       <c r="D25" s="6"/>
       <c r="E25" s="7" t="s">
@@ -6203,16 +6301,16 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="C27" s="50" t="s">
-        <v>465</v>
+        <v>475</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="3"/>
       <c r="B28" s="4" t="s">
-        <v>466</v>
+        <v>476</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>467</v>
+        <v>477</v>
       </c>
       <c r="D28" s="34" t="s">
         <v>260</v>
@@ -6224,10 +6322,10 @@
     <row r="29" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="3"/>
       <c r="B29" s="4" t="s">
-        <v>468</v>
+        <v>478</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>469</v>
+        <v>479</v>
       </c>
       <c r="D29" s="34" t="s">
         <v>260</v>
@@ -6302,7 +6400,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="59" t="s">
-        <v>470</v>
+        <v>480</v>
       </c>
       <c r="B1" s="52"/>
       <c r="C1" s="52"/>
@@ -6339,7 +6437,7 @@
     </row>
     <row r="4" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="60" t="s">
-        <v>471</v>
+        <v>481</v>
       </c>
       <c r="B4" s="52"/>
       <c r="C4" s="52"/>
@@ -6351,13 +6449,13 @@
         <v>6</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>472</v>
+        <v>482</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>473</v>
+        <v>483</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>474</v>
+        <v>484</v>
       </c>
       <c r="E5" s="7" t="s">
         <v>10</v>
@@ -6368,13 +6466,13 @@
         <v>6</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>475</v>
+        <v>485</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>476</v>
+        <v>486</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>477</v>
+        <v>487</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>10</v>
@@ -6385,13 +6483,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>478</v>
+        <v>488</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>479</v>
+        <v>489</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>480</v>
+        <v>490</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>10</v>
@@ -6402,13 +6500,13 @@
         <v>6</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>481</v>
+        <v>491</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>482</v>
+        <v>492</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>483</v>
+        <v>493</v>
       </c>
       <c r="E8" s="7" t="s">
         <v>10</v>
@@ -6419,13 +6517,13 @@
         <v>6</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>484</v>
+        <v>494</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>485</v>
+        <v>495</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>486</v>
+        <v>496</v>
       </c>
       <c r="E9" s="7" t="s">
         <v>10</v>
@@ -6436,13 +6534,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>487</v>
+        <v>497</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>488</v>
+        <v>498</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>489</v>
+        <v>499</v>
       </c>
       <c r="E10" s="7" t="s">
         <v>10</v>
@@ -6450,7 +6548,7 @@
     </row>
     <row r="12" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="60" t="s">
-        <v>490</v>
+        <v>500</v>
       </c>
       <c r="B12" s="52"/>
       <c r="C12" s="52"/>
@@ -6462,13 +6560,13 @@
         <v>6</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>491</v>
+        <v>501</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>492</v>
+        <v>502</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>493</v>
+        <v>503</v>
       </c>
       <c r="E13" s="7" t="s">
         <v>10</v>
@@ -6479,10 +6577,10 @@
         <v>6</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>494</v>
+        <v>504</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>495</v>
+        <v>505</v>
       </c>
       <c r="D14" s="10"/>
       <c r="E14" s="7" t="s">
@@ -6494,10 +6592,10 @@
         <v>6</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>496</v>
+        <v>506</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>497</v>
+        <v>507</v>
       </c>
       <c r="D15" s="6"/>
       <c r="E15" s="7" t="s">
@@ -6509,10 +6607,10 @@
         <v>6</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>498</v>
+        <v>508</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>499</v>
+        <v>509</v>
       </c>
       <c r="D16" s="10"/>
       <c r="E16" s="7" t="s">
@@ -6524,13 +6622,13 @@
         <v>6</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>500</v>
+        <v>510</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>501</v>
+        <v>511</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>502</v>
+        <v>512</v>
       </c>
       <c r="E17" s="7" t="s">
         <v>10</v>
@@ -6541,10 +6639,10 @@
         <v>6</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>503</v>
+        <v>513</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>504</v>
+        <v>514</v>
       </c>
       <c r="D18" s="10"/>
       <c r="E18" s="7" t="s">

</xml_diff>

<commit_message>
Document the submission dialog and add its QA rows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TownHall_Checklist (1).xlsx
+++ b/TownHall_Checklist (1).xlsx
@@ -2691,7 +2691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E156"/>
+  <dimension ref="A1:E160"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" style="52" min="1" max="1"/>
@@ -5737,7 +5737,7 @@
       </c>
       <c r="C154" s="5" t="inlineStr">
         <is>
-          <t>Approve a report with a 3-paragraph note. On the tester's home (/tester), the report card shows a "Note from the builder" block with the first three lines — not a one-line fragment cut off with "…".</t>
+          <t>Approve a report with a long (3-paragraph) note and a 4-star rating. On /tester the card stays its usual height and shows "★★★★☆ 4/5 · Note from the builder" — the note text itself is not on the card.</t>
         </is>
       </c>
       <c r="D154" s="6" t="inlineStr">
@@ -5784,6 +5784,82 @@
         </is>
       </c>
       <c r="E156" s="7" t="n"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="3" t="n"/>
+      <c r="B157" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.19-4</t>
+        </is>
+      </c>
+      <c r="C157" s="5" t="inlineStr">
+        <is>
+          <t>Click that card: a dialog opens with status, "4 out of 5" with stars, submitted and reviewed dates, the whole note (scrolls inside the dialog, page behind does not move), the screenshots and "Open the mission →". Esc, the × and a click outside each close it; focus returns to the card.</t>
+        </is>
+      </c>
+      <c r="D157" s="6" t="inlineStr">
+        <is>
+          <t>New in tester home fixes</t>
+        </is>
+      </c>
+      <c r="E157" s="7" t="n"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="3" t="n"/>
+      <c r="B158" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.19-5</t>
+        </is>
+      </c>
+      <c r="C158" s="5" t="inlineStr">
+        <is>
+          <t>With 7+ submissions, My Submissions shows 6 and "Page 1 of 2"; Next shows the rest, Previous goes back. Switching filter (All / Pending / Approved) returns to page 1. With 6 or fewer there is no pager.</t>
+        </is>
+      </c>
+      <c r="D158" s="6" t="inlineStr">
+        <is>
+          <t>New in tester home fixes</t>
+        </is>
+      </c>
+      <c r="E158" s="7" t="n"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="3" t="n"/>
+      <c r="B159" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.19-6</t>
+        </is>
+      </c>
+      <c r="C159" s="5" t="inlineStr">
+        <is>
+          <t>New missions on /tester lists only live missions: as a builder, save a mission as a draft → it does not appear for a tester; publish it → it appears at the top. A mission that closes when full disappears from the strip.</t>
+        </is>
+      </c>
+      <c r="D159" s="6" t="inlineStr">
+        <is>
+          <t>New in tester home fixes</t>
+        </is>
+      </c>
+      <c r="E159" s="7" t="n"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="3" t="n"/>
+      <c r="B160" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.19-7</t>
+        </is>
+      </c>
+      <c r="C160" s="5" t="inlineStr">
+        <is>
+          <t>Both themes and 360px width: the dialog fits with a 16px gutter, its backdrop is dark in light mode too, and the card's rating and note tag wrap cleanly.</t>
+        </is>
+      </c>
+      <c r="D160" s="6" t="inlineStr">
+        <is>
+          <t>New in tester home fixes</t>
+        </is>
+      </c>
+      <c r="E160" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>

<commit_message>
Drop Browse Missions from the tester's top bar
The top bar gave testers a Voltage Browse Missions button while Tester
Home has its own, two primary CTAs in one view. The bar now carries a
CTA for builders only (New Project). Tester Home loses Update Profile;
settings stays one click away on the avatar.

The Explore tour's "Submit your own work" step pointed at the bar's
button, which for a tester read Browse Missions while the step said
New Project. With the button gone it would point at nothing, so the
step goes too.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TownHall_Checklist (1).xlsx
+++ b/TownHall_Checklist (1).xlsx
@@ -2691,7 +2691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E160"/>
+  <dimension ref="A1:E161"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" style="52" min="1" max="1"/>
@@ -5860,6 +5860,25 @@
         </is>
       </c>
       <c r="E160" s="7" t="n"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="3" t="n"/>
+      <c r="B161" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.19-8</t>
+        </is>
+      </c>
+      <c r="C161" s="5" t="inlineStr">
+        <is>
+          <t>As a tester, the top bar has search and your avatar but no Browse Missions button, on desktop and on mobile; Tester Home shows a single Browse Missions button and no Update Profile. The Explore tour runs without a step pointing at a missing button. As a builder, New Project is still in the top bar.</t>
+        </is>
+      </c>
+      <c r="D161" s="6" t="inlineStr">
+        <is>
+          <t>New in tester home fixes</t>
+        </is>
+      </c>
+      <c r="E161" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>

<commit_message>
Document the mission preview
Spec, the CLAUDE.md rule that the preview composes the tester's own
components and never AuditLogForm, and QA rows 2.20.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TownHall_Checklist (1).xlsx
+++ b/TownHall_Checklist (1).xlsx
@@ -2691,7 +2691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E161"/>
+  <dimension ref="A1:E169"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" style="52" min="1" max="1"/>
@@ -2883,7 +2883,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="19.5" customHeight="1" s="52">
       <c r="A11" s="55" t="inlineStr">
         <is>
@@ -3022,7 +3021,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="19.5" customHeight="1" s="52">
       <c r="A18" s="55" t="inlineStr">
         <is>
@@ -3192,7 +3190,6 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
     <row r="26" ht="19.5" customHeight="1" s="52">
       <c r="A26" s="55" t="inlineStr">
         <is>
@@ -3354,7 +3351,6 @@
         </is>
       </c>
     </row>
-    <row r="33"/>
     <row r="34" ht="19.5" customHeight="1" s="52">
       <c r="A34" s="55" t="inlineStr">
         <is>
@@ -3443,7 +3439,6 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
     <row r="39" ht="19.5" customHeight="1" s="52">
       <c r="A39" s="55" t="inlineStr">
         <is>
@@ -3528,7 +3523,6 @@
         </is>
       </c>
     </row>
-    <row r="43"/>
     <row r="44" ht="19.5" customHeight="1" s="52">
       <c r="A44" s="55" t="inlineStr">
         <is>
@@ -3775,7 +3769,6 @@
         </is>
       </c>
     </row>
-    <row r="54"/>
     <row r="55" ht="19.5" customHeight="1" s="52">
       <c r="A55" s="55" t="inlineStr">
         <is>
@@ -3891,7 +3884,6 @@
         </is>
       </c>
     </row>
-    <row r="60"/>
     <row r="61">
       <c r="A61" s="55" t="n"/>
       <c r="C61" t="inlineStr">
@@ -4237,7 +4229,6 @@
       </c>
       <c r="E76" s="7" t="n"/>
     </row>
-    <row r="77"/>
     <row r="78">
       <c r="A78" s="55" t="n"/>
       <c r="C78" t="inlineStr">
@@ -4591,7 +4582,6 @@
         </is>
       </c>
     </row>
-    <row r="94"/>
     <row r="95">
       <c r="A95" s="55" t="n"/>
       <c r="C95" t="inlineStr">
@@ -4899,7 +4889,6 @@
         </is>
       </c>
     </row>
-    <row r="109"/>
     <row r="110">
       <c r="A110" s="55" t="n"/>
       <c r="C110" t="inlineStr">
@@ -5720,7 +5709,7 @@
         </is>
       </c>
     </row>
-    <row r="153">
+    <row r="153" s="52">
       <c r="A153" s="55" t="n"/>
       <c r="C153" t="inlineStr">
         <is>
@@ -5728,7 +5717,7 @@
         </is>
       </c>
     </row>
-    <row r="154">
+    <row r="154" s="52">
       <c r="A154" s="3" t="n"/>
       <c r="B154" s="4" t="inlineStr">
         <is>
@@ -5879,6 +5868,147 @@
         </is>
       </c>
       <c r="E161" s="7" t="n"/>
+    </row>
+    <row r="162" s="52">
+      <c r="A162" s="55" t="n"/>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2.20 Mission preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" s="52">
+      <c r="A163" s="3" t="n"/>
+      <c r="B163" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.20-1</t>
+        </is>
+      </c>
+      <c r="C163" s="5" t="inlineStr">
+        <is>
+          <t>On New Mission, add a title and two steps without saving and press Preview: a dialog titled "What testers see" shows the title, project card, chips, the steps and, under "Work through the test case", each step with its answer buttons. Close, edit a step, Preview again → the edit shows. The project still has no new mission or draft.</t>
+        </is>
+      </c>
+      <c r="D163" s="6" t="inlineStr">
+        <is>
+          <t>New in mission preview</t>
+        </is>
+      </c>
+      <c r="E163" s="7" t="n"/>
+    </row>
+    <row r="164" s="52">
+      <c r="A164" s="3" t="n"/>
+      <c r="B164" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.20-2</t>
+        </is>
+      </c>
+      <c r="C164" s="5" t="inlineStr">
+        <is>
+          <t>Preview a UI / Design mission → every step shows "What you saw" with "Required — at least N characters" and Clear / Unclear / Couldn't tell. Process Flow and Component show Pass / Fail / Blocked and no "What you saw".</t>
+        </is>
+      </c>
+      <c r="D164" s="6" t="inlineStr">
+        <is>
+          <t>New in mission preview</t>
+        </is>
+      </c>
+      <c r="E164" s="7" t="n"/>
+    </row>
+    <row r="165" s="52">
+      <c r="A165" s="3" t="n"/>
+      <c r="B165" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.20-3</t>
+        </is>
+      </c>
+      <c r="C165" s="5" t="inlineStr">
+        <is>
+          <t>Inside the preview nothing responds: clicking Pass or a textarea does nothing, Tab moves only between ×, the Phone/Desktop toggle and Back to editing. Esc, × and a click outside close it and focus returns to Preview.</t>
+        </is>
+      </c>
+      <c r="D165" s="6" t="inlineStr">
+        <is>
+          <t>New in mission preview</t>
+        </is>
+      </c>
+      <c r="E165" s="7" t="n"/>
+    </row>
+    <row r="166" s="52">
+      <c r="A166" s="3" t="n"/>
+      <c r="B166" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.20-4</t>
+        </is>
+      </c>
+      <c r="C166" s="5" t="inlineStr">
+        <is>
+          <t>DevTools → Application → Local Storage: open, use and close the preview → no twnhall:audit-log:* key appears. Then Save as Draft → the saved mission matches the editor; the request carries no entries.* fields.</t>
+        </is>
+      </c>
+      <c r="D166" s="6" t="inlineStr">
+        <is>
+          <t>New in mission preview</t>
+        </is>
+      </c>
+      <c r="E166" s="7" t="n"/>
+    </row>
+    <row r="167" s="52">
+      <c r="A167" s="3" t="n"/>
+      <c r="B167" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.20-5</t>
+        </is>
+      </c>
+      <c r="C167" s="5" t="inlineStr">
+        <is>
+          <t>Device Mobile → the preview is a 360px-wide frame. Both → a Phone / Desktop toggle, Phone first. Desktop → full width, no toggle.</t>
+        </is>
+      </c>
+      <c r="D167" s="6" t="inlineStr">
+        <is>
+          <t>New in mission preview</t>
+        </is>
+      </c>
+      <c r="E167" s="7" t="n"/>
+    </row>
+    <row r="168" s="52">
+      <c r="A168" s="3" t="n"/>
+      <c r="B168" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.20-6</t>
+        </is>
+      </c>
+      <c r="C168" s="5" t="inlineStr">
+        <is>
+          <t>Leave a step's "What should happen" empty and Preview → a line above the frame says that step isn't finished and is left out; the rest render. With no steps at all → "No steps yet — follow the brief above." and no answer section.</t>
+        </is>
+      </c>
+      <c r="D168" s="6" t="inlineStr">
+        <is>
+          <t>New in mission preview</t>
+        </is>
+      </c>
+      <c r="E168" s="7" t="n"/>
+    </row>
+    <row r="169" s="52">
+      <c r="A169" s="3" t="n"/>
+      <c r="B169" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.20-7</t>
+        </is>
+      </c>
+      <c r="C169" s="5" t="inlineStr">
+        <is>
+          <t>Edit Mission on a live mission has the same Preview button. Both themes and 360px: the dialog fits with an 8px gutter, scrolls inside, and the backdrop is dark in light mode too.</t>
+        </is>
+      </c>
+      <c r="D169" s="6" t="inlineStr">
+        <is>
+          <t>New in mission preview</t>
+        </is>
+      </c>
+      <c r="E169" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>

<commit_message>
Describe the full-screen mission preview
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TownHall_Checklist (1).xlsx
+++ b/TownHall_Checklist (1).xlsx
@@ -5886,7 +5886,7 @@
       </c>
       <c r="C163" s="5" t="inlineStr">
         <is>
-          <t>On New Mission, add a title and two steps without saving and press Preview: a dialog titled "What testers see" shows the title, project card, chips, the steps and, under "Work through the test case", each step with its answer buttons. Close, edit a step, Preview again → the edit shows. The project still has no new mission or draft.</t>
+          <t>On New Mission, add a title and two steps without saving and press Preview: the whole screen becomes the tester's page — a top bar with Back to editing, "What testers see" and a Phone / Desktop toggle, and below it the title, project card, chips, steps and each step's answer buttons. Back, edit a step, Preview again → the edit shows. The project still has no new mission or draft.</t>
         </is>
       </c>
       <c r="D163" s="6" t="inlineStr">
@@ -5924,7 +5924,7 @@
       </c>
       <c r="C165" s="5" t="inlineStr">
         <is>
-          <t>Inside the preview nothing responds: clicking Pass or a textarea does nothing, Tab moves only between ×, the Phone/Desktop toggle and Back to editing. Esc, × and a click outside close it and focus returns to Preview.</t>
+          <t>Inside the preview nothing responds: clicking Pass or a textarea does nothing, Tab moves only between Back to editing and the Phone / Desktop toggle. Esc or Back closes it and focus returns to Preview.</t>
         </is>
       </c>
       <c r="D165" s="6" t="inlineStr">
@@ -5962,7 +5962,7 @@
       </c>
       <c r="C167" s="5" t="inlineStr">
         <is>
-          <t>Device Mobile → the preview is a 360px-wide frame. Both → a Phone / Desktop toggle, Phone first. Desktop → full width, no toggle.</t>
+          <t>Device Mobile or Both → the preview opens on Phone, a 360px frame. Device Desktop → it opens on Desktop. The toggle switches either way.</t>
         </is>
       </c>
       <c r="D167" s="6" t="inlineStr">
@@ -6000,7 +6000,7 @@
       </c>
       <c r="C169" s="5" t="inlineStr">
         <is>
-          <t>Edit Mission on a live mission has the same Preview button. Both themes and 360px: the dialog fits with an 8px gutter, scrolls inside, and the backdrop is dark in light mode too.</t>
+          <t>Edit Mission on a live mission has the same Preview button. Both themes, at 360px and desktop: the preview fills the screen, the page scrolls with no visible scrollbar and no second scroll area, and the form behind does not scroll.</t>
         </is>
       </c>
       <c r="D169" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Document doc navigation, the terms gate and the summary rule
CLAUDE.md: lib/docNav.ts is the one source for the long documents'
headings and nav; the terms gate names Terms and Privacy, never the
Guides; the summary's only length rule is the character cap.
lib/sentences.ts leaves the folder map. The spec records both
decisions, and the checklist gains QA rows for round 2.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TownHall_Checklist (1).xlsx
+++ b/TownHall_Checklist (1).xlsx
@@ -2691,7 +2691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E178"/>
+  <dimension ref="A1:E184"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" style="52" min="1" max="1"/>
@@ -6010,7 +6010,7 @@
       </c>
       <c r="E169" s="7" t="n"/>
     </row>
-    <row r="170">
+    <row r="170" s="52">
       <c r="A170" s="55" t="n"/>
       <c r="C170" t="inlineStr">
         <is>
@@ -6018,7 +6018,7 @@
         </is>
       </c>
     </row>
-    <row r="171">
+    <row r="171" s="52">
       <c r="A171" s="3" t="n"/>
       <c r="B171" s="4" t="inlineStr">
         <is>
@@ -6169,6 +6169,109 @@
         </is>
       </c>
       <c r="E178" s="7" t="n"/>
+    </row>
+    <row r="179" s="52">
+      <c r="A179" s="55" t="n"/>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2.22 Bug fix round 2 — terms gate, summary, doc nav, skills</t>
+        </is>
+      </c>
+    </row>
+    <row r="180" s="52">
+      <c r="A180" s="3" t="n"/>
+      <c r="B180" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.22-1</t>
+        </is>
+      </c>
+      <c r="C180" s="5" t="inlineStr">
+        <is>
+          <t>On /terms-accept the subhead and the checkbox name the Terms of Service and the Privacy Policy — never the Guides. Each link opens in a new tab and loads (no 404); the gate tab keeps its place.</t>
+        </is>
+      </c>
+      <c r="D180" s="6" t="inlineStr">
+        <is>
+          <t>New in bug fix round 2</t>
+        </is>
+      </c>
+      <c r="E180" s="7" t="n"/>
+    </row>
+    <row r="181" s="52">
+      <c r="A181" s="3" t="n"/>
+      <c r="B181" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.22-2</t>
+        </is>
+      </c>
+      <c r="C181" s="5" t="inlineStr">
+        <is>
+          <t>Create a project with a three-sentence summary under 200 characters → it saves. The label reads "What is it?" with no "(2 sentences)"; the counter still shows N / 200 and over 200 is still refused. Same on Edit Project.</t>
+        </is>
+      </c>
+      <c r="D181" s="6" t="inlineStr">
+        <is>
+          <t>New in bug fix round 2</t>
+        </is>
+      </c>
+      <c r="E181" s="7" t="n"/>
+    </row>
+    <row r="182" s="52">
+      <c r="A182" s="3" t="n"/>
+      <c r="B182" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.22-3</t>
+        </is>
+      </c>
+      <c r="C182" s="5" t="inlineStr">
+        <is>
+          <t>At 360px, open /terms, /privacy, /guides/builder and /guides/tester: an "On this page" block sits above the text, collapsed. Open it → sections and the four-document switcher; the current document says "(you are here)". No horizontal scroll, both themes.</t>
+        </is>
+      </c>
+      <c r="D182" s="6" t="inlineStr">
+        <is>
+          <t>New in bug fix round 2</t>
+        </is>
+      </c>
+      <c r="E182" s="7" t="n"/>
+    </row>
+    <row r="183" s="52">
+      <c r="A183" s="3" t="n"/>
+      <c r="B183" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.22-4</t>
+        </is>
+      </c>
+      <c r="C183" s="5" t="inlineStr">
+        <is>
+          <t>On desktop, the same four pages show a sticky sidebar beside the text. Pick a section with the keyboard (Tab, Enter) → the page jumps there, the URL gains #id, and the next Tab continues from that heading. With reduced motion on, the jump does not animate. A copied #id link opens at that section.</t>
+        </is>
+      </c>
+      <c r="D183" s="6" t="inlineStr">
+        <is>
+          <t>New in bug fix round 2</t>
+        </is>
+      </c>
+      <c r="E183" s="7" t="n"/>
+    </row>
+    <row r="184" s="52">
+      <c r="A184" s="3" t="n"/>
+      <c r="B184" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.22-5</t>
+        </is>
+      </c>
+      <c r="C184" s="5" t="inlineStr">
+        <is>
+          <t>Skills (verification and Settings): click or Enter a suggestion → the list closes and the caret stays in the input; typing reopens it. Arrow keys highlight a suggestion and Enter adds it; typing a custom skill and Enter adds that. Esc closes without adding. Add three skills without touching the mouse.</t>
+        </is>
+      </c>
+      <c r="D184" s="6" t="inlineStr">
+        <is>
+          <t>New in bug fix round 2</t>
+        </is>
+      </c>
+      <c r="E184" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>

<commit_message>
Remove the document switcher from the doc nav
The nav now lists only the current document's sections. The "Documents"
list, with its "(you are here)" marker, is gone by decision; the guides
link each other at their foot and the footer links all four. The
unused label field leaves lib/docNav.ts, and the test now asserts no
switcher renders.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TownHall_Checklist (1).xlsx
+++ b/TownHall_Checklist (1).xlsx
@@ -2883,6 +2883,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="19.5" customHeight="1" s="52">
       <c r="A11" s="55" t="inlineStr">
         <is>
@@ -3021,6 +3022,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="19.5" customHeight="1" s="52">
       <c r="A18" s="55" t="inlineStr">
         <is>
@@ -3190,6 +3192,7 @@
         </is>
       </c>
     </row>
+    <row r="25"/>
     <row r="26" ht="19.5" customHeight="1" s="52">
       <c r="A26" s="55" t="inlineStr">
         <is>
@@ -3351,6 +3354,7 @@
         </is>
       </c>
     </row>
+    <row r="33"/>
     <row r="34" ht="19.5" customHeight="1" s="52">
       <c r="A34" s="55" t="inlineStr">
         <is>
@@ -3439,6 +3443,7 @@
         </is>
       </c>
     </row>
+    <row r="38"/>
     <row r="39" ht="19.5" customHeight="1" s="52">
       <c r="A39" s="55" t="inlineStr">
         <is>
@@ -3523,6 +3528,7 @@
         </is>
       </c>
     </row>
+    <row r="43"/>
     <row r="44" ht="19.5" customHeight="1" s="52">
       <c r="A44" s="55" t="inlineStr">
         <is>
@@ -3769,6 +3775,7 @@
         </is>
       </c>
     </row>
+    <row r="54"/>
     <row r="55" ht="19.5" customHeight="1" s="52">
       <c r="A55" s="55" t="inlineStr">
         <is>
@@ -3884,6 +3891,7 @@
         </is>
       </c>
     </row>
+    <row r="60"/>
     <row r="61">
       <c r="A61" s="55" t="n"/>
       <c r="C61" t="inlineStr">
@@ -4229,6 +4237,7 @@
       </c>
       <c r="E76" s="7" t="n"/>
     </row>
+    <row r="77"/>
     <row r="78">
       <c r="A78" s="55" t="n"/>
       <c r="C78" t="inlineStr">
@@ -4582,6 +4591,7 @@
         </is>
       </c>
     </row>
+    <row r="94"/>
     <row r="95">
       <c r="A95" s="55" t="n"/>
       <c r="C95" t="inlineStr">
@@ -4889,6 +4899,7 @@
         </is>
       </c>
     </row>
+    <row r="109"/>
     <row r="110">
       <c r="A110" s="55" t="n"/>
       <c r="C110" t="inlineStr">
@@ -6225,7 +6236,7 @@
       </c>
       <c r="C182" s="5" t="inlineStr">
         <is>
-          <t>At 360px, open /terms, /privacy, /guides/builder and /guides/tester: an "On this page" block sits above the text, collapsed. Open it → sections and the four-document switcher; the current document says "(you are here)". No horizontal scroll, both themes.</t>
+          <t>At 360px, open /terms, /privacy, /guides/builder and /guides/tester: an "On this page" block sits above the text, collapsed. Open it → the document's sections only, no list of other documents. No horizontal scroll, both themes.</t>
         </is>
       </c>
       <c r="D182" s="6" t="inlineStr">

</xml_diff>

<commit_message>
test(report): model, rendered text, route; docs
- The model: agreement counts (one tester, even split, mixed), order,
  category labels, snapshots, legacy reports, the cap
- The rendered PDF, read back with pdfjs-dist: every step and tester
  present, no tester name, email or id anywhere in the text,
  screenshots on/off/broken, all missions in one document
- The route: owner filter, 404 for someone else's project, 413 at the
  caps without fetching, its own rate limit, filename and headers
- anonymity.test.mts covers lib/exportDb.ts and lib/report.ts

CLAUDE.md records the route, the caps and the react-pdf traps; the
shareable-report prompt is marked superseded; QA rows 2.23 added.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TownHall_Checklist (1).xlsx
+++ b/TownHall_Checklist (1).xlsx
@@ -2691,7 +2691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E184"/>
+  <dimension ref="A1:E191"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" style="52" min="1" max="1"/>
@@ -2883,7 +2883,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="19.5" customHeight="1" s="52">
       <c r="A11" s="55" t="inlineStr">
         <is>
@@ -3022,7 +3021,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="19.5" customHeight="1" s="52">
       <c r="A18" s="55" t="inlineStr">
         <is>
@@ -3192,7 +3190,6 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
     <row r="26" ht="19.5" customHeight="1" s="52">
       <c r="A26" s="55" t="inlineStr">
         <is>
@@ -3354,7 +3351,6 @@
         </is>
       </c>
     </row>
-    <row r="33"/>
     <row r="34" ht="19.5" customHeight="1" s="52">
       <c r="A34" s="55" t="inlineStr">
         <is>
@@ -3443,7 +3439,6 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
     <row r="39" ht="19.5" customHeight="1" s="52">
       <c r="A39" s="55" t="inlineStr">
         <is>
@@ -3528,7 +3523,6 @@
         </is>
       </c>
     </row>
-    <row r="43"/>
     <row r="44" ht="19.5" customHeight="1" s="52">
       <c r="A44" s="55" t="inlineStr">
         <is>
@@ -3775,7 +3769,6 @@
         </is>
       </c>
     </row>
-    <row r="54"/>
     <row r="55" ht="19.5" customHeight="1" s="52">
       <c r="A55" s="55" t="inlineStr">
         <is>
@@ -3891,7 +3884,6 @@
         </is>
       </c>
     </row>
-    <row r="60"/>
     <row r="61">
       <c r="A61" s="55" t="n"/>
       <c r="C61" t="inlineStr">
@@ -4237,7 +4229,6 @@
       </c>
       <c r="E76" s="7" t="n"/>
     </row>
-    <row r="77"/>
     <row r="78">
       <c r="A78" s="55" t="n"/>
       <c r="C78" t="inlineStr">
@@ -4591,7 +4582,6 @@
         </is>
       </c>
     </row>
-    <row r="94"/>
     <row r="95">
       <c r="A95" s="55" t="n"/>
       <c r="C95" t="inlineStr">
@@ -4899,7 +4889,6 @@
         </is>
       </c>
     </row>
-    <row r="109"/>
     <row r="110">
       <c r="A110" s="55" t="n"/>
       <c r="C110" t="inlineStr">
@@ -6283,6 +6272,128 @@
         </is>
       </c>
       <c r="E184" s="7" t="n"/>
+    </row>
+    <row r="185" s="52">
+      <c r="A185" s="55" t="n"/>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2.23 PDF report — Settings → Account → Export</t>
+        </is>
+      </c>
+    </row>
+    <row r="186" s="52">
+      <c r="A186" s="3" t="n"/>
+      <c r="B186" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.23-1</t>
+        </is>
+      </c>
+      <c r="C186" s="5" t="inlineStr">
+        <is>
+          <t>Pick a project and one mission with several reports, screenshots on → Download PDF. The file is named &lt;project&gt;-&lt;mission&gt;-report-&lt;date&gt;.pdf. Page one lists the steps by how many testers hit them, most first ("4 of 5 testers: Unclear"), then the status mix, rating and test case. Every page has the project · mission footer and "Page N of M".</t>
+        </is>
+      </c>
+      <c r="D186" s="6" t="inlineStr">
+        <is>
+          <t>New in PDF report</t>
+        </is>
+      </c>
+      <c r="E186" s="7" t="n"/>
+    </row>
+    <row r="187" s="52">
+      <c r="A187" s="3" t="n"/>
+      <c r="B187" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.23-2</t>
+        </is>
+      </c>
+      <c r="C187" s="5" t="inlineStr">
+        <is>
+          <t>Pick "All missions" → one PDF named &lt;project&gt;-all-missions-report-&lt;date&gt;.pdf: a contents page with each mission's top issue, then a section per mission. The CSV button beside it still downloads an Excel workbook.</t>
+        </is>
+      </c>
+      <c r="D187" s="6" t="inlineStr">
+        <is>
+          <t>New in PDF report</t>
+        </is>
+      </c>
+      <c r="E187" s="7" t="n"/>
+    </row>
+    <row r="188" s="52">
+      <c r="A188" s="3" t="n"/>
+      <c r="B188" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.23-3</t>
+        </is>
+      </c>
+      <c r="C188" s="5" t="inlineStr">
+        <is>
+          <t>Untick "Include screenshots in the PDF" and download again → no images anywhere, and no "Screenshot couldn't be included" lines. Tick it → each screenshot takes at most about a third of a page.</t>
+        </is>
+      </c>
+      <c r="D188" s="6" t="inlineStr">
+        <is>
+          <t>New in PDF report</t>
+        </is>
+      </c>
+      <c r="E188" s="7" t="n"/>
+    </row>
+    <row r="189" s="52">
+      <c r="A189" s="3" t="n"/>
+      <c r="B189" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.23-4</t>
+        </is>
+      </c>
+      <c r="C189" s="5" t="inlineStr">
+        <is>
+          <t>Open a downloaded PDF and search (Ctrl+F) for a tester's real name and email address → nothing found. Testers appear only as Tester 1, 2, 3, numbered the same as on the mission page.</t>
+        </is>
+      </c>
+      <c r="D189" s="6" t="inlineStr">
+        <is>
+          <t>New in PDF report</t>
+        </is>
+      </c>
+      <c r="E189" s="7" t="n"/>
+    </row>
+    <row r="190" s="52">
+      <c r="A190" s="3" t="n"/>
+      <c r="B190" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.23-5</t>
+        </is>
+      </c>
+      <c r="C190" s="5" t="inlineStr">
+        <is>
+          <t>A ui_design mission's PDF says Clear / Unclear / Couldn't tell; a process_flow mission's says Pass / Fail / Blocked. AI summaries sit in a tinted box labelled "AI-generated summary — written by a model".</t>
+        </is>
+      </c>
+      <c r="D190" s="6" t="inlineStr">
+        <is>
+          <t>New in PDF report</t>
+        </is>
+      </c>
+      <c r="E190" s="7" t="n"/>
+    </row>
+    <row r="191" s="52">
+      <c r="A191" s="3" t="n"/>
+      <c r="B191" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.23-6</t>
+        </is>
+      </c>
+      <c r="C191" s="5" t="inlineStr">
+        <is>
+          <t>A project or mission over the cap (more than 60 reports, or more than 40 screenshots with screenshots on) → the panel says, in its own alert, to choose a single mission or turn off screenshots. No file downloads. Downloading 6 PDFs inside an hour → the sixth says to try again later.</t>
+        </is>
+      </c>
+      <c r="D191" s="6" t="inlineStr">
+        <is>
+          <t>New in PDF report</t>
+        </is>
+      </c>
+      <c r="E191" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -6386,7 +6497,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E5:E9 E12:E16 E19:E24 E27:E32 E35:E37 E40:E42 E45:E53 E56:E59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E5:E9 E12:E16 E19:E24 E27:E32 E35:E37 E40:E42 E45:E53 E56:E59 E186 E187 E188 E189 E190 E191" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"To Do,In Progress,Done,Blocked,N/A"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
fix(report): name, log and count dropped screenshots
fetchOne returned null for four different reasons — off-bucket (the
SSRF guard), storage non-2xx, timeout or network, unsupported format —
all rendered as one caption, and nothing was logged. The format failure
behind the WebP bug was invisible for that reason.

Each now has a reason. The route logs it once per image with the report
id and never the URL. The caption says what happened, page one counts
what was left out, and X-Screenshots-Missing lets ExportPanel say so at
download. The SSRF guard is unchanged and still never fetches.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TownHall_Checklist (1).xlsx
+++ b/TownHall_Checklist (1).xlsx
@@ -2691,7 +2691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E191"/>
+  <dimension ref="A1:E194"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" style="52" min="1" max="1"/>
@@ -6328,7 +6328,7 @@
       </c>
       <c r="C188" s="5" t="inlineStr">
         <is>
-          <t>Untick "Include screenshots in the PDF" and download again → no images anywhere, and no "Screenshot couldn't be included" lines. Tick it → each screenshot takes at most about a third of a page.</t>
+          <t>Untick "Include screenshots in the PDF" and download again → no images anywhere, and no "Screenshot could not be loaded" or "format not supported" lines. Tick it → each screenshot takes at most about a third of a page.</t>
         </is>
       </c>
       <c r="D188" s="6" t="inlineStr">
@@ -6394,6 +6394,63 @@
         </is>
       </c>
       <c r="E191" s="7" t="n"/>
+    </row>
+    <row r="192" s="52">
+      <c r="A192" s="3" t="n"/>
+      <c r="B192" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.23-7</t>
+        </is>
+      </c>
+      <c r="C192" s="5" t="inlineStr">
+        <is>
+          <t>Submit a report with a WebP screenshot (any phone or browser upload — the form re-encodes most uploads to WebP), then Download PDF with screenshots on → the image is in the PDF. Check with `pdfimages -list &lt;file&gt;.pdf`, not by eye: the table lists one row per screenshot.</t>
+        </is>
+      </c>
+      <c r="D192" s="6" t="inlineStr">
+        <is>
+          <t>New in PDF screenshots fix</t>
+        </is>
+      </c>
+      <c r="E192" s="7" t="n"/>
+    </row>
+    <row r="193" s="52">
+      <c r="A193" s="3" t="n"/>
+      <c r="B193" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.23-8</t>
+        </is>
+      </c>
+      <c r="C193" s="5" t="inlineStr">
+        <is>
+          <t>A report filed before multiple screenshots (only the legacy screenshot_url set) → its screenshot appears in the PDF exactly as on the mission page, and the CSV's screenshot count includes it.</t>
+        </is>
+      </c>
+      <c r="D193" s="6" t="inlineStr">
+        <is>
+          <t>New in PDF screenshots fix</t>
+        </is>
+      </c>
+      <c r="E193" s="7" t="n"/>
+    </row>
+    <row r="194" s="52">
+      <c r="A194" s="3" t="n"/>
+      <c r="B194" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.23-9</t>
+        </is>
+      </c>
+      <c r="C194" s="5" t="inlineStr">
+        <is>
+          <t>Break one screenshot URL (delete the object in Storage) and Download PDF → in its place the PDF says "Screenshot could not be loaded.", page one says "1 of N screenshots couldn't be included", the panel says the same after download, and the Vercel log has "[export/report] screenshot left out" with reason "unavailable", HTTP 404 and the report id — no URL.</t>
+        </is>
+      </c>
+      <c r="D194" s="6" t="inlineStr">
+        <is>
+          <t>New in PDF screenshots fix</t>
+        </is>
+      </c>
+      <c r="E194" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>

<commit_message>
docs: three tiers in CLAUDE.md, the spec and the QA checklist
CLAUDE.md: three tiers, monthlyReports as the single source for the
allowance, prices written in both currencies and never computed.
Commits the compensation model's 22 October revision the tiers come
from.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TownHall_Checklist (1).xlsx
+++ b/TownHall_Checklist (1).xlsx
@@ -2691,7 +2691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E194"/>
+  <dimension ref="A1:E200"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" style="52" min="1" max="1"/>
@@ -6451,6 +6451,109 @@
         </is>
       </c>
       <c r="E194" s="7" t="n"/>
+    </row>
+    <row r="195" s="52">
+      <c r="A195" s="55" t="n"/>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2.24 Three tiers — Starter, and the naira price</t>
+        </is>
+      </c>
+    </row>
+    <row r="196" s="52">
+      <c r="A196" s="3" t="n"/>
+      <c r="B196" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.24-1</t>
+        </is>
+      </c>
+      <c r="C196" s="5" t="inlineStr">
+        <is>
+          <t>Read /pricing as a Nigerian founder: Starter ₦15,000 / month · ~$11, Pro ₦30,000 / month · ~$22, naira the large figure. No "₦10–12k", no "$19", no "best value" or highlighted tier. Calls to action are "Ask about Starter" / "Ask about Pro" → /contact, never Subscribe or Upgrade.</t>
+        </is>
+      </c>
+      <c r="D196" s="6" t="inlineStr">
+        <is>
+          <t>New in three tiers</t>
+        </is>
+      </c>
+      <c r="E196" s="7" t="n"/>
+    </row>
+    <row r="197" s="52">
+      <c r="A197" s="3" t="n"/>
+      <c r="B197" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.24-2</t>
+        </is>
+      </c>
+      <c r="C197" s="5" t="inlineStr">
+        <is>
+          <t>At 360px, both themes: /pricing shows Community, Starter, Pro stacked in that order with no horizontal scroll; Compare plans is a list, each feature followed by one line per plan. From 1024px the three cards sit side by side and the table has four columns.</t>
+        </is>
+      </c>
+      <c r="D197" s="6" t="inlineStr">
+        <is>
+          <t>New in three tiers</t>
+        </is>
+      </c>
+      <c r="E197" s="7" t="n"/>
+    </row>
+    <row r="198" s="52">
+      <c r="A198" s="3" t="n"/>
+      <c r="B198" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.24-3</t>
+        </is>
+      </c>
+      <c r="C198" s="5" t="inlineStr">
+        <is>
+          <t>Admin → Users: set a builder to Starter → the select shows Starter and "Recent plan and cohort changes" logs Community → Starter with your name. Set Pro, then Community → the column is cleared (null) and the account behaves as Community.</t>
+        </is>
+      </c>
+      <c r="D198" s="6" t="inlineStr">
+        <is>
+          <t>New in three tiers</t>
+        </is>
+      </c>
+      <c r="E198" s="7" t="n"/>
+    </row>
+    <row r="199" s="52">
+      <c r="A199" s="3" t="n"/>
+      <c r="B199" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.24-4</t>
+        </is>
+      </c>
+      <c r="C199" s="5" t="inlineStr">
+        <is>
+          <t>As that Starter builder, open a draft mission → the notice beside Publish says 5 reports available. Publish → the mission opens to 5 testers; the next draft says no reports available (5, not 10). Three live missions → a fourth is refused at the active-mission limit.</t>
+        </is>
+      </c>
+      <c r="D199" s="6" t="inlineStr">
+        <is>
+          <t>New in three tiers</t>
+        </is>
+      </c>
+      <c r="E199" s="7" t="n"/>
+    </row>
+    <row r="200" s="52">
+      <c r="A200" s="3" t="n"/>
+      <c r="B200" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.24-5</t>
+        </is>
+      </c>
+      <c r="C200" s="5" t="inlineStr">
+        <is>
+          <t>Settings → Plan on each of Community, Starter and Pro, at 360px and desktop: the plan you are on is first and labelled "Your plan", the other two follow with their naira and dollar prices. No usage meter, no upgrade button.</t>
+        </is>
+      </c>
+      <c r="D200" s="6" t="inlineStr">
+        <is>
+          <t>New in three tiers</t>
+        </is>
+      </c>
+      <c r="E200" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>

<commit_message>
docs: PDF plain language in CLAUDE.md, the spec and the QA checklist
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TownHall_Checklist (1).xlsx
+++ b/TownHall_Checklist (1).xlsx
@@ -2691,7 +2691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E200"/>
+  <dimension ref="A1:E207"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" style="52" min="1" max="1"/>
@@ -6295,7 +6295,7 @@
       </c>
       <c r="D186" s="6" t="inlineStr">
         <is>
-          <t>New in PDF report</t>
+          <t>RETEST - front reordered, ratings removed in feat/pdf-plain-language</t>
         </is>
       </c>
       <c r="E186" s="7" t="n"/>
@@ -6314,7 +6314,7 @@
       </c>
       <c r="D187" s="6" t="inlineStr">
         <is>
-          <t>New in PDF report</t>
+          <t>RETEST - front reordered, ratings removed in feat/pdf-plain-language</t>
         </is>
       </c>
       <c r="E187" s="7" t="n"/>
@@ -6554,6 +6554,128 @@
         </is>
       </c>
       <c r="E200" s="7" t="n"/>
+    </row>
+    <row r="201" s="52">
+      <c r="A201" s="55" t="n"/>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2.25 PDF report — readable by a non-technical reader</t>
+        </is>
+      </c>
+    </row>
+    <row r="202" s="52">
+      <c r="A202" s="3" t="n"/>
+      <c r="B202" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.25-1</t>
+        </is>
+      </c>
+      <c r="C202" s="5" t="inlineStr">
+        <is>
+          <t>Download a one-mission PDF and an all-missions PDF. Each opens, under the project name, with three or four plain sentences: how many people were asked to try the product, on what device, between which dates, how to read what follows, and the one place the word "mission" is explained. The rest of the document says "test".</t>
+        </is>
+      </c>
+      <c r="D202" s="6" t="inlineStr">
+        <is>
+          <t>New in PDF plain language</t>
+        </is>
+      </c>
+      <c r="E202" s="7" t="n"/>
+    </row>
+    <row r="203" s="52">
+      <c r="A203" s="3" t="n"/>
+      <c r="B203" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.25-2</t>
+        </is>
+      </c>
+      <c r="C203" s="5" t="inlineStr">
+        <is>
+          <t>Under "What we found", every step with a problem leads with a sentence ("Four of the five people said this did not come across the way it was meant to."), then "They were asked to: …", "What should have happened: …", and only then the small "Step 2 · 4 of 5 testers: Unclear" line.</t>
+        </is>
+      </c>
+      <c r="D203" s="6" t="inlineStr">
+        <is>
+          <t>New in PDF plain language</t>
+        </is>
+      </c>
+      <c r="E203" s="7" t="n"/>
+    </row>
+    <row r="204" s="52">
+      <c r="A204" s="3" t="n"/>
+      <c r="B204" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.25-3</t>
+        </is>
+      </c>
+      <c r="C204" s="5" t="inlineStr">
+        <is>
+          <t>"How each step was answered" quotes word for word what testers see beside the status buttons on /mission/[id]: Pass / Fail / Blocked hints on a process_flow mission, Clear / Unclear / Couldn't tell on a ui_design one, both sets (Pass first) in an all-missions PDF that holds both.</t>
+        </is>
+      </c>
+      <c r="D204" s="6" t="inlineStr">
+        <is>
+          <t>New in PDF plain language</t>
+        </is>
+      </c>
+      <c r="E204" s="7" t="n"/>
+    </row>
+    <row r="205" s="52">
+      <c r="A205" s="3" t="n"/>
+      <c r="B205" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.25-4</t>
+        </is>
+      </c>
+      <c r="C205" s="5" t="inlineStr">
+        <is>
+          <t>Print page one in greyscale (or set the printer to black and white): beside each finding, one dot per tester — filled where they hit a problem, hollow where not — still clearly readable, with the written count beside it.</t>
+        </is>
+      </c>
+      <c r="D205" s="6" t="inlineStr">
+        <is>
+          <t>New in PDF plain language</t>
+        </is>
+      </c>
+      <c r="E205" s="7" t="n"/>
+    </row>
+    <row r="206" s="52">
+      <c r="A206" s="3" t="n"/>
+      <c r="B206" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.25-5</t>
+        </is>
+      </c>
+      <c r="C206" s="5" t="inlineStr">
+        <is>
+          <t>Search the PDF (Ctrl+F) for "rating", "rated" and "/ 5" → nothing found, on a mission whose reports the builder has rated. The last page, "What the words mean", explains only words that appear earlier in that document.</t>
+        </is>
+      </c>
+      <c r="D206" s="6" t="inlineStr">
+        <is>
+          <t>New in PDF plain language</t>
+        </is>
+      </c>
+      <c r="E206" s="7" t="n"/>
+    </row>
+    <row r="207" s="52">
+      <c r="A207" s="3" t="n"/>
+      <c r="B207" s="4" t="inlineStr">
+        <is>
+          <t>QA-2.25-6</t>
+        </is>
+      </c>
+      <c r="C207" s="5" t="inlineStr">
+        <is>
+          <t>Give a five-tester PDF to someone with no technical background. From the first two pages alone they can say what was tested and by whom, and name the three things the builder should fix. Record their answers in docs/specs/SPEC-pdf-plain-language.md §7.</t>
+        </is>
+      </c>
+      <c r="D207" s="6" t="inlineStr">
+        <is>
+          <t>New in PDF plain language</t>
+        </is>
+      </c>
+      <c r="E207" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>